<commit_message>
updated ore veins langs and sheet
</commit_message>
<xml_diff>
--- a/OresToFieldGuide/data/sheet.xlsx
+++ b/OresToFieldGuide/data/sheet.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="500" uniqueCount="500">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="499" uniqueCount="499">
   <si>
     <t>Vein ID</t>
   </si>
@@ -1004,16 +1004,13 @@
     <t>moon_desh</t>
   </si>
   <si>
-    <t>desh: 40 [2]</t>
-  </si>
-  <si>
-    <t>ilmenite: 25 [1]</t>
-  </si>
-  <si>
-    <t>aluminium: 20</t>
-  </si>
-  <si>
-    <t>armalcolite: 15</t>
+    <t>desh: 25 [2]</t>
+  </si>
+  <si>
+    <t>ilmenite: 30 [1]</t>
+  </si>
+  <si>
+    <t>aluminium: 25</t>
   </si>
   <si>
     <t>moon_garnet</t>
@@ -4121,7 +4118,7 @@
         <v>10</v>
       </c>
       <c r="G27" s="3">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="J27" s="3" t="s">
         <v>146</v>
@@ -8821,7 +8818,7 @@
         <v>200</v>
       </c>
       <c r="D3" s="3">
-        <v>0.4</v>
+        <v>0.35</v>
       </c>
       <c r="E3" s="3">
         <v>0</v>
@@ -8830,7 +8827,7 @@
         <v>80</v>
       </c>
       <c r="G3" s="3">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="J3" s="3" t="s">
         <v>315</v>
@@ -8883,7 +8880,7 @@
         <v>260</v>
       </c>
       <c r="D4" s="3">
-        <v>0.45</v>
+        <v>0.35</v>
       </c>
       <c r="E4" s="3">
         <v>0</v>
@@ -8895,7 +8892,7 @@
         <v>70</v>
       </c>
       <c r="I4" s="3">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="J4" s="3" t="s">
         <v>319</v>
@@ -8963,7 +8960,7 @@
         <v>128</v>
       </c>
       <c r="G5" s="3">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="J5" s="3" t="s">
         <v>323</v>
@@ -9093,7 +9090,7 @@
         <v>80</v>
       </c>
       <c r="G7" s="3">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="J7" s="3" t="s">
         <v>329</v>
@@ -9105,7 +9102,7 @@
         <v>331</v>
       </c>
       <c r="M7" s="3" t="s">
-        <v>332</v>
+        <v>317</v>
       </c>
       <c r="O7" s="1" t="s">
         <v>36</v>
@@ -9140,7 +9137,7 @@
     </row>
     <row r="8">
       <c r="A8" s="3" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>38</v>
@@ -9164,16 +9161,16 @@
         <v>7</v>
       </c>
       <c r="J8" s="3" t="s">
+        <v>333</v>
+      </c>
+      <c r="K8" s="3" t="s">
         <v>334</v>
       </c>
-      <c r="K8" s="3" t="s">
+      <c r="L8" s="3" t="s">
         <v>335</v>
       </c>
-      <c r="L8" s="3" t="s">
+      <c r="M8" s="3" t="s">
         <v>336</v>
-      </c>
-      <c r="M8" s="3" t="s">
-        <v>337</v>
       </c>
       <c r="O8" s="1" t="s">
         <v>36</v>
@@ -9208,7 +9205,7 @@
     </row>
     <row r="9">
       <c r="A9" s="3" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>31</v>
@@ -9217,7 +9214,7 @@
         <v>250</v>
       </c>
       <c r="D9" s="3">
-        <v>0.4</v>
+        <v>0.35</v>
       </c>
       <c r="E9" s="3">
         <v>5</v>
@@ -9226,7 +9223,7 @@
         <v>85</v>
       </c>
       <c r="G9" s="3">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="J9" s="3" t="s">
         <v>276</v>
@@ -9238,7 +9235,7 @@
         <v>125</v>
       </c>
       <c r="M9" s="3" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="N9" s="3" t="s">
         <v>127</v>
@@ -9276,7 +9273,7 @@
     </row>
     <row r="10">
       <c r="A10" s="3" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>38</v>
@@ -9285,7 +9282,7 @@
         <v>170</v>
       </c>
       <c r="D10" s="3">
-        <v>0.4</v>
+        <v>0.35</v>
       </c>
       <c r="E10" s="3">
         <v>10</v>
@@ -9294,7 +9291,7 @@
         <v>80</v>
       </c>
       <c r="G10" s="3">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="H10" s="3">
         <v>10</v>
@@ -9306,7 +9303,7 @@
         <v>268</v>
       </c>
       <c r="L10" s="3" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="M10" s="3" t="s">
         <v>131</v>
@@ -9344,7 +9341,7 @@
     </row>
     <row r="11">
       <c r="A11" s="3" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>99</v>
@@ -9353,7 +9350,7 @@
         <v>260</v>
       </c>
       <c r="D11" s="3">
-        <v>0.55</v>
+        <v>0.4</v>
       </c>
       <c r="E11" s="3">
         <v>0</v>
@@ -9365,16 +9362,16 @@
         <v>60</v>
       </c>
       <c r="I11" s="3">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="J11" s="3" t="s">
+        <v>342</v>
+      </c>
+      <c r="K11" s="3" t="s">
         <v>343</v>
       </c>
-      <c r="K11" s="3" t="s">
+      <c r="L11" s="3" t="s">
         <v>344</v>
-      </c>
-      <c r="L11" s="3" t="s">
-        <v>345</v>
       </c>
       <c r="O11" s="2" t="s">
         <v>35</v>
@@ -9409,7 +9406,7 @@
     </row>
     <row r="12">
       <c r="A12" s="3" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>38</v>
@@ -9427,7 +9424,7 @@
         <v>100</v>
       </c>
       <c r="G12" s="3">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="H12" s="3">
         <v>9</v>
@@ -9436,13 +9433,13 @@
         <v>137</v>
       </c>
       <c r="K12" s="3" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="L12" s="3" t="s">
         <v>202</v>
       </c>
       <c r="M12" s="3" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="N12" s="3" t="s">
         <v>313</v>
@@ -9480,7 +9477,7 @@
     </row>
     <row r="13">
       <c r="A13" s="3" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>31</v>
@@ -9498,7 +9495,7 @@
         <v>66</v>
       </c>
       <c r="G13" s="3">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="J13" s="3" t="s">
         <v>154</v>
@@ -9548,7 +9545,7 @@
     </row>
     <row r="14">
       <c r="A14" s="3" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>31</v>
@@ -9557,7 +9554,7 @@
         <v>280</v>
       </c>
       <c r="D14" s="3">
-        <v>0.3</v>
+        <v>0.25</v>
       </c>
       <c r="E14" s="3">
         <v>0</v>
@@ -9566,16 +9563,16 @@
         <v>90</v>
       </c>
       <c r="G14" s="3">
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="J14" s="3" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="K14" s="3" t="s">
         <v>63</v>
       </c>
       <c r="L14" s="3" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="M14" s="3" t="s">
         <v>65</v>
@@ -9616,7 +9613,7 @@
     </row>
     <row r="15">
       <c r="A15" s="3" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>31</v>
@@ -9625,7 +9622,7 @@
         <v>215</v>
       </c>
       <c r="D15" s="3">
-        <v>0.5</v>
+        <v>0.35</v>
       </c>
       <c r="E15" s="3">
         <v>5</v>
@@ -9634,7 +9631,7 @@
         <v>80</v>
       </c>
       <c r="G15" s="3">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="J15" s="3" t="s">
         <v>165</v>
@@ -9681,7 +9678,7 @@
     </row>
     <row r="16">
       <c r="A16" s="3" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>31</v>
@@ -9702,7 +9699,7 @@
         <v>35</v>
       </c>
       <c r="J16" s="3" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="K16" s="3" t="s">
         <v>171</v>
@@ -9711,7 +9708,7 @@
         <v>172</v>
       </c>
       <c r="M16" s="3" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="N16" s="3" t="s">
         <v>313</v>
@@ -9749,7 +9746,7 @@
     </row>
     <row r="17">
       <c r="A17" s="3" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>31</v>
@@ -9758,7 +9755,7 @@
         <v>245</v>
       </c>
       <c r="D17" s="3">
-        <v>0.45</v>
+        <v>0.35</v>
       </c>
       <c r="E17" s="3">
         <v>0</v>
@@ -9767,7 +9764,7 @@
         <v>50</v>
       </c>
       <c r="G17" s="3">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="J17" s="3" t="s">
         <v>68</v>
@@ -9814,7 +9811,7 @@
     </row>
     <row r="18">
       <c r="A18" s="3" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>31</v>
@@ -9832,7 +9829,7 @@
         <v>70</v>
       </c>
       <c r="G18" s="3">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="J18" s="3" t="s">
         <v>274</v>
@@ -9844,7 +9841,7 @@
         <v>177</v>
       </c>
       <c r="M18" s="3" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="O18" s="1" t="s">
         <v>36</v>
@@ -9879,7 +9876,7 @@
     </row>
     <row r="19">
       <c r="A19" s="3" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>31</v>
@@ -9897,19 +9894,19 @@
         <v>80</v>
       </c>
       <c r="G19" s="3">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="J19" s="3" t="s">
+        <v>360</v>
+      </c>
+      <c r="K19" s="3" t="s">
         <v>361</v>
       </c>
-      <c r="K19" s="3" t="s">
+      <c r="L19" s="3" t="s">
         <v>362</v>
       </c>
-      <c r="L19" s="3" t="s">
+      <c r="M19" s="3" t="s">
         <v>363</v>
-      </c>
-      <c r="M19" s="3" t="s">
-        <v>364</v>
       </c>
       <c r="O19" s="1" t="s">
         <v>36</v>
@@ -9944,7 +9941,7 @@
     </row>
     <row r="20">
       <c r="A20" s="3" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>31</v>
@@ -9962,19 +9959,19 @@
         <v>100</v>
       </c>
       <c r="G20" s="3">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="J20" s="3" t="s">
+        <v>365</v>
+      </c>
+      <c r="K20" s="3" t="s">
         <v>366</v>
       </c>
-      <c r="K20" s="3" t="s">
+      <c r="L20" s="3" t="s">
         <v>367</v>
       </c>
-      <c r="L20" s="3" t="s">
+      <c r="M20" s="3" t="s">
         <v>368</v>
-      </c>
-      <c r="M20" s="3" t="s">
-        <v>369</v>
       </c>
       <c r="O20" s="1" t="s">
         <v>36</v>
@@ -10009,7 +10006,7 @@
     </row>
     <row r="21">
       <c r="A21" s="3" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>31</v>
@@ -10027,7 +10024,7 @@
         <v>100</v>
       </c>
       <c r="G21" s="3">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="J21" s="3" t="s">
         <v>190</v>
@@ -10074,7 +10071,7 @@
     </row>
     <row r="22">
       <c r="A22" s="3" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>31</v>
@@ -10092,19 +10089,19 @@
         <v>90</v>
       </c>
       <c r="G22" s="3">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="J22" s="3" t="s">
+        <v>371</v>
+      </c>
+      <c r="K22" s="3" t="s">
         <v>372</v>
       </c>
-      <c r="K22" s="3" t="s">
+      <c r="L22" s="3" t="s">
         <v>373</v>
       </c>
-      <c r="L22" s="3" t="s">
+      <c r="M22" s="3" t="s">
         <v>374</v>
-      </c>
-      <c r="M22" s="3" t="s">
-        <v>375</v>
       </c>
       <c r="O22" s="1" t="s">
         <v>36</v>
@@ -10139,7 +10136,7 @@
     </row>
     <row r="23">
       <c r="A23" s="3" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>38</v>
@@ -10175,7 +10172,7 @@
         <v>79</v>
       </c>
       <c r="N23" s="3" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="O23" s="2" t="s">
         <v>35</v>
@@ -10210,7 +10207,7 @@
     </row>
     <row r="24">
       <c r="A24" s="3" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>31</v>
@@ -10219,7 +10216,7 @@
         <v>200</v>
       </c>
       <c r="D24" s="3">
-        <v>0.45</v>
+        <v>0.4</v>
       </c>
       <c r="E24" s="3">
         <v>0</v>
@@ -10231,13 +10228,13 @@
         <v>20</v>
       </c>
       <c r="J24" s="3" t="s">
+        <v>378</v>
+      </c>
+      <c r="K24" s="3" t="s">
         <v>379</v>
       </c>
-      <c r="K24" s="3" t="s">
+      <c r="L24" s="3" t="s">
         <v>380</v>
-      </c>
-      <c r="L24" s="3" t="s">
-        <v>381</v>
       </c>
       <c r="O24" s="2" t="s">
         <v>35</v>
@@ -10272,7 +10269,7 @@
     </row>
     <row r="25">
       <c r="A25" s="3" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>31</v>
@@ -10281,7 +10278,7 @@
         <v>210</v>
       </c>
       <c r="D25" s="3">
-        <v>0.4</v>
+        <v>0.35</v>
       </c>
       <c r="E25" s="3">
         <v>20</v>
@@ -10296,7 +10293,7 @@
         <v>204</v>
       </c>
       <c r="K25" s="3" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="L25" s="3" t="s">
         <v>265</v>
@@ -10337,7 +10334,7 @@
     </row>
     <row r="26">
       <c r="A26" s="3" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="B26" s="3" t="s">
         <v>31</v>
@@ -10346,7 +10343,7 @@
         <v>205</v>
       </c>
       <c r="D26" s="3">
-        <v>0.4</v>
+        <v>0.35</v>
       </c>
       <c r="E26" s="3">
         <v>2</v>
@@ -10355,13 +10352,13 @@
         <v>75</v>
       </c>
       <c r="G26" s="3">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="J26" s="3" t="s">
+        <v>384</v>
+      </c>
+      <c r="K26" s="3" t="s">
         <v>385</v>
-      </c>
-      <c r="K26" s="3" t="s">
-        <v>386</v>
       </c>
       <c r="L26" s="3" t="s">
         <v>217</v>
@@ -10399,7 +10396,7 @@
     </row>
     <row r="27">
       <c r="A27" s="3" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="B27" s="3" t="s">
         <v>31</v>
@@ -10417,19 +10414,19 @@
         <v>128</v>
       </c>
       <c r="G27" s="3">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="J27" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="K27" s="3" t="s">
         <v>388</v>
-      </c>
-      <c r="K27" s="3" t="s">
-        <v>389</v>
       </c>
       <c r="L27" s="3" t="s">
         <v>222</v>
       </c>
       <c r="M27" s="3" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="O27" s="1" t="s">
         <v>36</v>
@@ -10464,7 +10461,7 @@
     </row>
     <row r="28">
       <c r="A28" s="3" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="B28" s="3" t="s">
         <v>38</v>
@@ -10473,7 +10470,7 @@
         <v>210</v>
       </c>
       <c r="D28" s="3">
-        <v>0.5</v>
+        <v>0.35</v>
       </c>
       <c r="E28" s="3">
         <v>0</v>
@@ -10482,10 +10479,10 @@
         <v>120</v>
       </c>
       <c r="G28" s="3">
-        <v>64</v>
+        <v>45</v>
       </c>
       <c r="H28" s="3">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="J28" s="3" t="s">
         <v>85</v>
@@ -10622,16 +10619,16 @@
         <v>11</v>
       </c>
       <c r="P1" s="4" t="s">
+        <v>391</v>
+      </c>
+      <c r="Q1" s="4" t="s">
         <v>392</v>
-      </c>
-      <c r="Q1" s="4" t="s">
-        <v>393</v>
       </c>
       <c r="R1" s="4" t="s">
         <v>17</v>
       </c>
       <c r="S1" s="4" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="T1" s="4" t="s">
         <v>19</v>
@@ -10648,7 +10645,7 @@
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>38</v>
@@ -10672,7 +10669,7 @@
         <v>4</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="O2" s="2" t="s">
         <v>35</v>
@@ -10704,7 +10701,7 @@
     </row>
     <row r="3">
       <c r="A3" s="3" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>31</v>
@@ -10725,10 +10722,10 @@
         <v>39</v>
       </c>
       <c r="J3" s="3" t="s">
+        <v>397</v>
+      </c>
+      <c r="K3" s="3" t="s">
         <v>398</v>
-      </c>
-      <c r="K3" s="3" t="s">
-        <v>399</v>
       </c>
       <c r="L3" s="3" t="s">
         <v>92</v>
@@ -10763,7 +10760,7 @@
     </row>
     <row r="4">
       <c r="A4" s="3" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>38</v>
@@ -10787,13 +10784,13 @@
         <v>9</v>
       </c>
       <c r="J4" s="3" t="s">
+        <v>400</v>
+      </c>
+      <c r="K4" s="3" t="s">
         <v>401</v>
       </c>
-      <c r="K4" s="3" t="s">
+      <c r="L4" s="3" t="s">
         <v>402</v>
-      </c>
-      <c r="L4" s="3" t="s">
-        <v>403</v>
       </c>
       <c r="M4" s="3" t="s">
         <v>97</v>
@@ -10828,7 +10825,7 @@
     </row>
     <row r="5">
       <c r="A5" s="3" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>99</v>
@@ -10893,7 +10890,7 @@
     </row>
     <row r="6">
       <c r="A6" s="3" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>31</v>
@@ -10914,10 +10911,10 @@
         <v>45</v>
       </c>
       <c r="J6" s="3" t="s">
+        <v>405</v>
+      </c>
+      <c r="K6" s="3" t="s">
         <v>406</v>
-      </c>
-      <c r="K6" s="3" t="s">
-        <v>407</v>
       </c>
       <c r="O6" s="2" t="s">
         <v>35</v>
@@ -10949,7 +10946,7 @@
     </row>
     <row r="7">
       <c r="A7" s="3" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>31</v>
@@ -11011,7 +11008,7 @@
     </row>
     <row r="8">
       <c r="A8" s="3" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>31</v>
@@ -11032,16 +11029,16 @@
         <v>45</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="K8" s="3" t="s">
         <v>114</v>
       </c>
       <c r="L8" s="3" t="s">
+        <v>410</v>
+      </c>
+      <c r="M8" s="3" t="s">
         <v>411</v>
-      </c>
-      <c r="M8" s="3" t="s">
-        <v>412</v>
       </c>
       <c r="O8" s="1" t="s">
         <v>36</v>
@@ -11073,7 +11070,7 @@
     </row>
     <row r="9">
       <c r="A9" s="3" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>38</v>
@@ -11097,16 +11094,16 @@
         <v>8</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="K9" s="3" t="s">
         <v>40</v>
       </c>
       <c r="L9" s="3" t="s">
+        <v>414</v>
+      </c>
+      <c r="M9" s="3" t="s">
         <v>415</v>
-      </c>
-      <c r="M9" s="3" t="s">
-        <v>416</v>
       </c>
       <c r="O9" s="1" t="s">
         <v>36</v>
@@ -11138,7 +11135,7 @@
     </row>
     <row r="10">
       <c r="A10" s="3" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>31</v>
@@ -11159,13 +11156,13 @@
         <v>45</v>
       </c>
       <c r="J10" s="3" t="s">
+        <v>417</v>
+      </c>
+      <c r="K10" s="3" t="s">
         <v>418</v>
       </c>
-      <c r="K10" s="3" t="s">
+      <c r="L10" s="3" t="s">
         <v>419</v>
-      </c>
-      <c r="L10" s="3" t="s">
-        <v>420</v>
       </c>
       <c r="M10" s="3" t="s">
         <v>121</v>
@@ -11200,7 +11197,7 @@
     </row>
     <row r="11">
       <c r="A11" s="3" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>31</v>
@@ -11227,10 +11224,10 @@
         <v>277</v>
       </c>
       <c r="L11" s="3" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="M11" s="3" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="N11" s="3" t="s">
         <v>127</v>
@@ -11265,7 +11262,7 @@
     </row>
     <row r="12">
       <c r="A12" s="3" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>31</v>
@@ -11286,10 +11283,10 @@
         <v>37</v>
       </c>
       <c r="J12" s="3" t="s">
+        <v>423</v>
+      </c>
+      <c r="K12" s="3" t="s">
         <v>424</v>
-      </c>
-      <c r="K12" s="3" t="s">
-        <v>425</v>
       </c>
       <c r="L12" s="3" t="s">
         <v>49</v>
@@ -11327,7 +11324,7 @@
     </row>
     <row r="13">
       <c r="A13" s="3" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>31</v>
@@ -11389,7 +11386,7 @@
     </row>
     <row r="14">
       <c r="A14" s="3" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>99</v>
@@ -11413,13 +11410,13 @@
         <v>12</v>
       </c>
       <c r="J14" s="3" t="s">
+        <v>427</v>
+      </c>
+      <c r="K14" s="3" t="s">
         <v>428</v>
       </c>
-      <c r="K14" s="3" t="s">
+      <c r="L14" s="3" t="s">
         <v>429</v>
-      </c>
-      <c r="L14" s="3" t="s">
-        <v>430</v>
       </c>
       <c r="O14" s="2" t="s">
         <v>35</v>
@@ -11451,7 +11448,7 @@
     </row>
     <row r="15">
       <c r="A15" s="3" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>38</v>
@@ -11475,16 +11472,16 @@
         <v>9</v>
       </c>
       <c r="J15" s="3" t="s">
+        <v>431</v>
+      </c>
+      <c r="K15" s="3" t="s">
         <v>432</v>
-      </c>
-      <c r="K15" s="3" t="s">
-        <v>433</v>
       </c>
       <c r="L15" s="3" t="s">
         <v>139</v>
       </c>
       <c r="M15" s="3" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="O15" s="2" t="s">
         <v>35</v>
@@ -11516,7 +11513,7 @@
     </row>
     <row r="16">
       <c r="A16" s="3" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>31</v>
@@ -11543,7 +11540,7 @@
         <v>53</v>
       </c>
       <c r="L16" s="3" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="M16" s="3" t="s">
         <v>55</v>
@@ -11581,7 +11578,7 @@
     </row>
     <row r="17">
       <c r="A17" s="3" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>31</v>
@@ -11602,13 +11599,13 @@
         <v>40</v>
       </c>
       <c r="J17" s="3" t="s">
+        <v>436</v>
+      </c>
+      <c r="K17" s="3" t="s">
         <v>437</v>
       </c>
-      <c r="K17" s="3" t="s">
+      <c r="L17" s="3" t="s">
         <v>438</v>
-      </c>
-      <c r="L17" s="3" t="s">
-        <v>439</v>
       </c>
       <c r="M17" s="3" t="s">
         <v>149</v>
@@ -11643,7 +11640,7 @@
     </row>
     <row r="18">
       <c r="A18" s="3" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>31</v>
@@ -11667,13 +11664,13 @@
         <v>272</v>
       </c>
       <c r="K18" s="3" t="s">
+        <v>440</v>
+      </c>
+      <c r="L18" s="3" t="s">
         <v>441</v>
       </c>
-      <c r="L18" s="3" t="s">
+      <c r="M18" s="3" t="s">
         <v>442</v>
-      </c>
-      <c r="M18" s="3" t="s">
-        <v>443</v>
       </c>
       <c r="N18" s="3" t="s">
         <v>158</v>
@@ -11708,7 +11705,7 @@
     </row>
     <row r="19">
       <c r="A19" s="3" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>31</v>
@@ -11729,16 +11726,16 @@
         <v>39</v>
       </c>
       <c r="J19" s="3" t="s">
+        <v>444</v>
+      </c>
+      <c r="K19" s="3" t="s">
         <v>445</v>
-      </c>
-      <c r="K19" s="3" t="s">
-        <v>446</v>
       </c>
       <c r="L19" s="3" t="s">
         <v>163</v>
       </c>
       <c r="M19" s="3" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="N19" s="3" t="s">
         <v>66</v>
@@ -11773,7 +11770,7 @@
     </row>
     <row r="20">
       <c r="A20" s="3" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>31</v>
@@ -11797,10 +11794,10 @@
         <v>290</v>
       </c>
       <c r="K20" s="3" t="s">
+        <v>448</v>
+      </c>
+      <c r="L20" s="3" t="s">
         <v>449</v>
-      </c>
-      <c r="L20" s="3" t="s">
-        <v>450</v>
       </c>
       <c r="M20" s="3" t="s">
         <v>168</v>
@@ -11835,7 +11832,7 @@
     </row>
     <row r="21">
       <c r="A21" s="3" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>31</v>
@@ -11856,13 +11853,13 @@
         <v>41</v>
       </c>
       <c r="J21" s="3" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="K21" s="3" t="s">
+        <v>451</v>
+      </c>
+      <c r="L21" s="3" t="s">
         <v>452</v>
-      </c>
-      <c r="L21" s="3" t="s">
-        <v>453</v>
       </c>
       <c r="O21" s="2" t="s">
         <v>35</v>
@@ -11894,7 +11891,7 @@
     </row>
     <row r="22">
       <c r="A22" s="3" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>31</v>
@@ -11921,10 +11918,10 @@
         <v>69</v>
       </c>
       <c r="L22" s="3" t="s">
+        <v>454</v>
+      </c>
+      <c r="M22" s="3" t="s">
         <v>455</v>
-      </c>
-      <c r="M22" s="3" t="s">
-        <v>456</v>
       </c>
       <c r="O22" s="2" t="s">
         <v>35</v>
@@ -11956,7 +11953,7 @@
     </row>
     <row r="23">
       <c r="A23" s="3" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>31</v>
@@ -11977,13 +11974,13 @@
         <v>45</v>
       </c>
       <c r="J23" s="3" t="s">
+        <v>457</v>
+      </c>
+      <c r="K23" s="3" t="s">
         <v>458</v>
       </c>
-      <c r="K23" s="3" t="s">
+      <c r="L23" s="3" t="s">
         <v>459</v>
-      </c>
-      <c r="L23" s="3" t="s">
-        <v>460</v>
       </c>
       <c r="O23" s="2" t="s">
         <v>35</v>
@@ -12015,7 +12012,7 @@
     </row>
     <row r="24">
       <c r="A24" s="3" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>31</v>
@@ -12036,7 +12033,7 @@
         <v>32</v>
       </c>
       <c r="J24" s="3" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="O24" s="1" t="s">
         <v>36</v>
@@ -12068,7 +12065,7 @@
     </row>
     <row r="25">
       <c r="A25" s="3" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>31</v>
@@ -12089,13 +12086,13 @@
         <v>31</v>
       </c>
       <c r="J25" s="3" t="s">
+        <v>463</v>
+      </c>
+      <c r="K25" s="3" t="s">
         <v>464</v>
       </c>
-      <c r="K25" s="3" t="s">
+      <c r="L25" s="3" t="s">
         <v>465</v>
-      </c>
-      <c r="L25" s="3" t="s">
-        <v>466</v>
       </c>
       <c r="M25" s="3" t="s">
         <v>184</v>
@@ -12130,7 +12127,7 @@
     </row>
     <row r="26">
       <c r="A26" s="3" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="B26" s="3" t="s">
         <v>31</v>
@@ -12189,7 +12186,7 @@
     </row>
     <row r="27">
       <c r="A27" s="3" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="B27" s="3" t="s">
         <v>31</v>
@@ -12210,13 +12207,13 @@
         <v>45</v>
       </c>
       <c r="J27" s="3" t="s">
+        <v>468</v>
+      </c>
+      <c r="K27" s="3" t="s">
         <v>469</v>
       </c>
-      <c r="K27" s="3" t="s">
+      <c r="L27" s="3" t="s">
         <v>470</v>
-      </c>
-      <c r="L27" s="3" t="s">
-        <v>471</v>
       </c>
       <c r="O27" s="1" t="s">
         <v>36</v>
@@ -12248,7 +12245,7 @@
     </row>
     <row r="28">
       <c r="A28" s="3" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="B28" s="3" t="s">
         <v>31</v>
@@ -12272,10 +12269,10 @@
         <v>190</v>
       </c>
       <c r="K28" s="3" t="s">
+        <v>472</v>
+      </c>
+      <c r="L28" s="3" t="s">
         <v>473</v>
-      </c>
-      <c r="L28" s="3" t="s">
-        <v>474</v>
       </c>
       <c r="O28" s="2" t="s">
         <v>35</v>
@@ -12307,7 +12304,7 @@
     </row>
     <row r="29">
       <c r="A29" s="3" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="B29" s="3" t="s">
         <v>31</v>
@@ -12328,13 +12325,13 @@
         <v>50</v>
       </c>
       <c r="J29" s="3" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="K29" s="3" t="s">
+        <v>475</v>
+      </c>
+      <c r="L29" s="3" t="s">
         <v>476</v>
-      </c>
-      <c r="L29" s="3" t="s">
-        <v>477</v>
       </c>
       <c r="M29" s="3" t="s">
         <v>202</v>
@@ -12369,7 +12366,7 @@
     </row>
     <row r="30">
       <c r="A30" s="3" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="B30" s="3" t="s">
         <v>38</v>
@@ -12399,10 +12396,10 @@
         <v>77</v>
       </c>
       <c r="L30" s="3" t="s">
+        <v>478</v>
+      </c>
+      <c r="M30" s="3" t="s">
         <v>479</v>
-      </c>
-      <c r="M30" s="3" t="s">
-        <v>480</v>
       </c>
       <c r="O30" s="2" t="s">
         <v>35</v>
@@ -12434,7 +12431,7 @@
     </row>
     <row r="31">
       <c r="A31" s="3" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="B31" s="3" t="s">
         <v>31</v>
@@ -12455,13 +12452,13 @@
         <v>25</v>
       </c>
       <c r="J31" s="3" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="K31" s="3" t="s">
         <v>82</v>
       </c>
       <c r="L31" s="3" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="O31" s="2" t="s">
         <v>35</v>
@@ -12493,7 +12490,7 @@
     </row>
     <row r="32">
       <c r="A32" s="3" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="B32" s="3" t="s">
         <v>31</v>
@@ -12517,10 +12514,10 @@
         <v>264</v>
       </c>
       <c r="K32" s="3" t="s">
+        <v>484</v>
+      </c>
+      <c r="L32" s="3" t="s">
         <v>485</v>
-      </c>
-      <c r="L32" s="3" t="s">
-        <v>486</v>
       </c>
       <c r="O32" s="2" t="s">
         <v>35</v>
@@ -12552,7 +12549,7 @@
     </row>
     <row r="33">
       <c r="A33" s="3" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="B33" s="3" t="s">
         <v>31</v>
@@ -12573,13 +12570,13 @@
         <v>45</v>
       </c>
       <c r="J33" s="3" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="K33" s="3" t="s">
         <v>209</v>
       </c>
       <c r="L33" s="3" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="O33" s="1" t="s">
         <v>36</v>
@@ -12611,7 +12608,7 @@
     </row>
     <row r="34">
       <c r="A34" s="3" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="B34" s="3" t="s">
         <v>31</v>
@@ -12632,13 +12629,13 @@
         <v>50</v>
       </c>
       <c r="J34" s="3" t="s">
+        <v>490</v>
+      </c>
+      <c r="K34" s="3" t="s">
         <v>491</v>
       </c>
-      <c r="K34" s="3" t="s">
+      <c r="L34" s="3" t="s">
         <v>492</v>
-      </c>
-      <c r="L34" s="3" t="s">
-        <v>493</v>
       </c>
       <c r="O34" s="1" t="s">
         <v>36</v>
@@ -12670,7 +12667,7 @@
     </row>
     <row r="35">
       <c r="A35" s="3" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="B35" s="3" t="s">
         <v>31</v>
@@ -12691,7 +12688,7 @@
         <v>17</v>
       </c>
       <c r="J35" s="3" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="O35" s="2" t="s">
         <v>35</v>
@@ -12723,7 +12720,7 @@
     </row>
     <row r="36">
       <c r="A36" s="3" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="B36" s="3" t="s">
         <v>31</v>
@@ -12744,10 +12741,10 @@
         <v>45</v>
       </c>
       <c r="J36" s="3" t="s">
+        <v>496</v>
+      </c>
+      <c r="K36" s="3" t="s">
         <v>497</v>
-      </c>
-      <c r="K36" s="3" t="s">
-        <v>498</v>
       </c>
       <c r="L36" s="3" t="s">
         <v>222</v>
@@ -12782,7 +12779,7 @@
     </row>
     <row r="37">
       <c r="A37" s="3" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="B37" s="3" t="s">
         <v>38</v>

</xml_diff>

<commit_message>
added visual vein info for two venus veins
</commit_message>
<xml_diff>
--- a/OresToFieldGuide/data/sheet.xlsx
+++ b/OresToFieldGuide/data/sheet.xlsx
@@ -9,13 +9,14 @@
     <sheet name="mars" sheetId="2" r:id="rId3"/>
     <sheet name="moon" sheetId="3" r:id="rId4"/>
     <sheet name="nether" sheetId="4" r:id="rId5"/>
+    <sheet name="venus" sheetId="5" r:id="rId6"/>
   </sheets>
   <calcPr fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="514" uniqueCount="514">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="519" uniqueCount="519">
   <si>
     <t>Vein ID</t>
   </si>
@@ -1557,6 +1558,21 @@
   </si>
   <si>
     <t>nether_topaz</t>
+  </si>
+  <si>
+    <t>venus_manual_salt</t>
+  </si>
+  <si>
+    <t>salt: 50</t>
+  </si>
+  <si>
+    <t>spodumene: 15</t>
+  </si>
+  <si>
+    <t>venus_manual_sulfur</t>
+  </si>
+  <si>
+    <t>sulfur: 50</t>
   </si>
 </sst>
 </file>
@@ -13096,4 +13112,218 @@
   </sheetData>
   <headerFooter/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:U3"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="20.293367385864258" customWidth="1" style="3"/>
+    <col min="2" max="2" width="14.972405433654785" customWidth="1" style="3"/>
+    <col min="3" max="3" width="9.140625" customWidth="1" style="3"/>
+    <col min="4" max="4" width="9.140625" customWidth="1" style="3"/>
+    <col min="5" max="5" width="9.140625" customWidth="1" style="3"/>
+    <col min="6" max="6" width="9.140625" customWidth="1" style="3"/>
+    <col min="7" max="7" width="9.140625" customWidth="1" style="3"/>
+    <col min="8" max="8" width="9.140625" customWidth="1" style="3"/>
+    <col min="9" max="9" width="9.140625" customWidth="1" style="3"/>
+    <col min="10" max="10" width="9.682135581970215" customWidth="1" style="3"/>
+    <col min="11" max="11" width="12.619355201721191" customWidth="1" style="3"/>
+    <col min="12" max="12" width="13.423484802246094" customWidth="1" style="3"/>
+    <col min="13" max="13" width="15.053228378295898" customWidth="1" style="3"/>
+    <col min="14" max="14" width="9.140625" customWidth="1" style="3"/>
+    <col min="15" max="15" width="9.140625" customWidth="1" style="3"/>
+    <col min="16" max="16" width="9.140625" customWidth="1" style="3"/>
+    <col min="17" max="17" width="9.140625" customWidth="1" style="3"/>
+    <col min="18" max="18" width="9.140625" customWidth="1" style="3"/>
+    <col min="19" max="19" width="10.040207862854004" customWidth="1" style="3"/>
+    <col min="20" max="20" width="9.140625" customWidth="1" style="3"/>
+    <col min="21" max="21" width="12.787137985229492" customWidth="1" style="3"/>
+    <col min="22" max="22" width="9.140625" customWidth="1" style="3"/>
+    <col min="23" max="23" width="9.140625" customWidth="1" style="3"/>
+    <col min="24" max="24" width="9.140625" customWidth="1" style="3"/>
+    <col min="25" max="25" width="9.140625" customWidth="1" style="3"/>
+    <col min="26" max="26" width="9.140625" customWidth="1" style="3"/>
+    <col min="27" max="27" width="9.140625" customWidth="1" style="3"/>
+    <col min="28" max="28" width="9.140625" customWidth="1" style="3"/>
+    <col min="29" max="29" width="9.140625" customWidth="1" style="3"/>
+    <col min="30" max="30" width="9.140625" customWidth="1" style="3"/>
+    <col min="31" max="31" width="9.140625" customWidth="1" style="3"/>
+    <col min="32" max="32" width="9.140625" customWidth="1" style="3"/>
+    <col min="33" max="33" width="9.140625" customWidth="1" style="3"/>
+    <col min="34" max="34" width="9.140625" customWidth="1" style="3"/>
+    <col min="35" max="35" width="9.140625" customWidth="1" style="3"/>
+    <col min="36" max="36" width="9.140625" customWidth="1" style="3"/>
+    <col min="37" max="37" width="9.140625" customWidth="1" style="3"/>
+    <col min="38" max="38" width="9.140625" customWidth="1" style="3"/>
+    <col min="39" max="39" width="9.140625" customWidth="1" style="3"/>
+    <col min="40" max="40" width="9.140625" customWidth="1" style="3"/>
+    <col min="41" max="41" width="9.140625" customWidth="1" style="3"/>
+    <col min="42" max="42" width="9.140625" customWidth="1" style="3"/>
+    <col min="43" max="43" width="9.140625" customWidth="1" style="3"/>
+    <col min="44" max="44" width="9.140625" customWidth="1" style="3"/>
+    <col min="45" max="45" width="9.140625" customWidth="1" style="3"/>
+    <col min="46" max="16384" width="9.140625" customWidth="1" style="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" s="4" customFormat="1">
+      <c r="A1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="P1" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="Q1" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="R1" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="S1" s="4" t="s">
+        <v>407</v>
+      </c>
+      <c r="T1" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="U1" s="4" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="s">
+        <v>514</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C2" s="3">
+        <v>100</v>
+      </c>
+      <c r="D2" s="3">
+        <v>0.2</v>
+      </c>
+      <c r="E2" s="3">
+        <v>40</v>
+      </c>
+      <c r="F2" s="3">
+        <v>65</v>
+      </c>
+      <c r="G2" s="3">
+        <v>20</v>
+      </c>
+      <c r="H2" s="3">
+        <v>6</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>515</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>214</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>198</v>
+      </c>
+      <c r="M2" s="3" t="s">
+        <v>516</v>
+      </c>
+      <c r="P2" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="Q2" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="R2" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="S2" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="T2" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="U2" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="s">
+        <v>517</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C3" s="3">
+        <v>100</v>
+      </c>
+      <c r="D3" s="3">
+        <v>0.2</v>
+      </c>
+      <c r="E3" s="3">
+        <v>40</v>
+      </c>
+      <c r="F3" s="3">
+        <v>65</v>
+      </c>
+      <c r="G3" s="3">
+        <v>15</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>518</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="L3" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="P3" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="Q3" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="R3" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="S3" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="T3" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="U3" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+  </sheetData>
+  <headerFooter/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
add lapis to mars
</commit_message>
<xml_diff>
--- a/OresToFieldGuide/data/sheet.xlsx
+++ b/OresToFieldGuide/data/sheet.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="523" uniqueCount="523">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="524" uniqueCount="524">
   <si>
     <t>Vein ID</t>
   </si>
@@ -856,6 +856,9 @@
   </si>
   <si>
     <t>mars_hematite</t>
+  </si>
+  <si>
+    <t>mars_lapis</t>
   </si>
   <si>
     <t>mars_lubricant</t>
@@ -6438,7 +6441,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AF28"/>
+  <dimension ref="A1:AF29"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="26.277278900146484" customWidth="1" style="3"/>
@@ -7609,7 +7612,7 @@
         <v>31</v>
       </c>
       <c r="C14" s="3">
-        <v>220</v>
+        <v>200</v>
       </c>
       <c r="D14" s="3">
         <v>0.25</v>
@@ -7621,25 +7624,19 @@
         <v>70</v>
       </c>
       <c r="G14" s="3">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="J14" s="3" t="s">
-        <v>281</v>
+        <v>148</v>
       </c>
       <c r="K14" s="3" t="s">
-        <v>282</v>
+        <v>149</v>
       </c>
       <c r="L14" s="3" t="s">
-        <v>283</v>
+        <v>150</v>
       </c>
       <c r="M14" s="3" t="s">
-        <v>284</v>
-      </c>
-      <c r="N14" s="3" t="s">
-        <v>285</v>
-      </c>
-      <c r="O14" s="3" t="s">
-        <v>116</v>
+        <v>151</v>
       </c>
       <c r="P14" s="2" t="s">
         <v>35</v>
@@ -7647,23 +7644,23 @@
       <c r="Q14" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="R14" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="S14" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="T14" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="U14" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="V14" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="W14" s="1" t="s">
-        <v>36</v>
+      <c r="R14" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="S14" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="T14" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="U14" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="V14" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="W14" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="X14" s="1" t="s">
         <v>36</v>
@@ -7671,8 +7668,8 @@
       <c r="Y14" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="Z14" s="1" t="s">
-        <v>36</v>
+      <c r="Z14" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="AA14" s="1" t="s">
         <v>36</v>
@@ -7680,8 +7677,8 @@
       <c r="AB14" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="AC14" s="1" t="s">
-        <v>36</v>
+      <c r="AC14" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="AD14" s="2" t="s">
         <v>35</v>
@@ -7695,16 +7692,16 @@
     </row>
     <row r="15">
       <c r="A15" s="3" t="s">
-        <v>286</v>
+        <v>281</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>31</v>
       </c>
       <c r="C15" s="3">
-        <v>215</v>
+        <v>220</v>
       </c>
       <c r="D15" s="3">
-        <v>0.4</v>
+        <v>0.25</v>
       </c>
       <c r="E15" s="3">
         <v>0</v>
@@ -7713,40 +7710,46 @@
         <v>70</v>
       </c>
       <c r="G15" s="3">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="J15" s="3" t="s">
-        <v>287</v>
+        <v>282</v>
       </c>
       <c r="K15" s="3" t="s">
-        <v>178</v>
+        <v>283</v>
       </c>
       <c r="L15" s="3" t="s">
-        <v>179</v>
+        <v>284</v>
       </c>
       <c r="M15" s="3" t="s">
+        <v>285</v>
+      </c>
+      <c r="N15" s="3" t="s">
+        <v>286</v>
+      </c>
+      <c r="O15" s="3" t="s">
         <v>116</v>
       </c>
       <c r="P15" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="Q15" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="R15" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="S15" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="T15" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="U15" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="V15" s="2" t="s">
-        <v>35</v>
+      <c r="Q15" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="R15" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="S15" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="T15" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="U15" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="V15" s="1" t="s">
+        <v>36</v>
       </c>
       <c r="W15" s="1" t="s">
         <v>36</v>
@@ -7754,40 +7757,40 @@
       <c r="X15" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="Y15" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="Z15" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="AA15" s="2" t="s">
-        <v>35</v>
+      <c r="Y15" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="Z15" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AA15" s="1" t="s">
+        <v>36</v>
       </c>
       <c r="AB15" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="AC15" s="2" t="s">
-        <v>35</v>
+      <c r="AC15" s="1" t="s">
+        <v>36</v>
       </c>
       <c r="AD15" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="AE15" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="AF15" s="1" t="s">
-        <v>36</v>
+      <c r="AE15" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AF15" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>31</v>
       </c>
       <c r="C16" s="3">
-        <v>250</v>
+        <v>215</v>
       </c>
       <c r="D16" s="3">
         <v>0.4</v>
@@ -7799,16 +7802,16 @@
         <v>70</v>
       </c>
       <c r="G16" s="3">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="J16" s="3" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="K16" s="3" t="s">
-        <v>290</v>
+        <v>178</v>
       </c>
       <c r="L16" s="3" t="s">
-        <v>127</v>
+        <v>179</v>
       </c>
       <c r="M16" s="3" t="s">
         <v>116</v>
@@ -7822,61 +7825,61 @@
       <c r="R16" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="S16" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="T16" s="1" t="s">
-        <v>36</v>
+      <c r="S16" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="T16" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="U16" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="V16" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="W16" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="X16" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="Y16" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="Z16" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="AA16" s="1" t="s">
-        <v>36</v>
+      <c r="V16" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="W16" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="X16" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="Y16" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="Z16" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="AA16" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="AB16" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="AC16" s="1" t="s">
-        <v>36</v>
+      <c r="AC16" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="AD16" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="AE16" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="AF16" s="2" t="s">
-        <v>35</v>
+      <c r="AE16" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="AF16" s="1" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>31</v>
       </c>
       <c r="C17" s="3">
-        <v>220</v>
+        <v>250</v>
       </c>
       <c r="D17" s="3">
-        <v>0.55</v>
+        <v>0.4</v>
       </c>
       <c r="E17" s="3">
         <v>0</v>
@@ -7885,52 +7888,55 @@
         <v>70</v>
       </c>
       <c r="G17" s="3">
-        <v>20</v>
+        <v>55</v>
       </c>
       <c r="J17" s="3" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="K17" s="3" t="s">
-        <v>253</v>
+        <v>291</v>
       </c>
       <c r="L17" s="3" t="s">
-        <v>293</v>
+        <v>127</v>
+      </c>
+      <c r="M17" s="3" t="s">
+        <v>116</v>
       </c>
       <c r="P17" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="Q17" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="R17" s="2" t="s">
-        <v>35</v>
+      <c r="Q17" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="R17" s="1" t="s">
+        <v>36</v>
       </c>
       <c r="S17" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="T17" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="U17" s="1" t="s">
-        <v>36</v>
+      <c r="T17" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="U17" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="V17" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="W17" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="X17" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="Y17" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="Z17" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="AA17" s="2" t="s">
-        <v>35</v>
+      <c r="W17" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="X17" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="Y17" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="Z17" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AA17" s="1" t="s">
+        <v>36</v>
       </c>
       <c r="AB17" s="1" t="s">
         <v>36</v>
@@ -7944,22 +7950,22 @@
       <c r="AE17" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="AF17" s="1" t="s">
-        <v>36</v>
+      <c r="AF17" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>31</v>
       </c>
       <c r="C18" s="3">
-        <v>210</v>
+        <v>220</v>
       </c>
       <c r="D18" s="3">
-        <v>0.3</v>
+        <v>0.55</v>
       </c>
       <c r="E18" s="3">
         <v>0</v>
@@ -7968,19 +7974,16 @@
         <v>70</v>
       </c>
       <c r="G18" s="3">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="J18" s="3" t="s">
-        <v>188</v>
+        <v>293</v>
       </c>
       <c r="K18" s="3" t="s">
-        <v>189</v>
+        <v>253</v>
       </c>
       <c r="L18" s="3" t="s">
-        <v>190</v>
-      </c>
-      <c r="M18" s="3" t="s">
-        <v>116</v>
+        <v>294</v>
       </c>
       <c r="P18" s="2" t="s">
         <v>35</v>
@@ -7988,35 +7991,35 @@
       <c r="Q18" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="R18" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="S18" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="T18" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="U18" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="V18" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="W18" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="X18" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="Y18" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="Z18" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="AA18" s="1" t="s">
-        <v>36</v>
+      <c r="R18" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="S18" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="T18" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="U18" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="V18" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="W18" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="X18" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="Y18" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="Z18" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="AA18" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="AB18" s="1" t="s">
         <v>36</v>
@@ -8039,13 +8042,13 @@
         <v>295</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="C19" s="3">
         <v>210</v>
       </c>
       <c r="D19" s="3">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="E19" s="3">
         <v>0</v>
@@ -8056,20 +8059,17 @@
       <c r="G19" s="3">
         <v>40</v>
       </c>
-      <c r="H19" s="3">
-        <v>6</v>
-      </c>
       <c r="J19" s="3" t="s">
-        <v>296</v>
+        <v>188</v>
       </c>
       <c r="K19" s="3" t="s">
-        <v>215</v>
+        <v>189</v>
       </c>
       <c r="L19" s="3" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
       <c r="M19" s="3" t="s">
-        <v>216</v>
+        <v>116</v>
       </c>
       <c r="P19" s="2" t="s">
         <v>35</v>
@@ -8092,8 +8092,8 @@
       <c r="V19" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="W19" s="1" t="s">
-        <v>36</v>
+      <c r="W19" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="X19" s="2" t="s">
         <v>35</v>
@@ -8116,8 +8116,8 @@
       <c r="AD19" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="AE19" s="2" t="s">
-        <v>35</v>
+      <c r="AE19" s="1" t="s">
+        <v>36</v>
       </c>
       <c r="AF19" s="1" t="s">
         <v>36</v>
@@ -8125,10 +8125,10 @@
     </row>
     <row r="20">
       <c r="A20" s="3" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="C20" s="3">
         <v>210</v>
@@ -8145,23 +8145,26 @@
       <c r="G20" s="3">
         <v>40</v>
       </c>
+      <c r="H20" s="3">
+        <v>6</v>
+      </c>
       <c r="J20" s="3" t="s">
-        <v>225</v>
+        <v>297</v>
       </c>
       <c r="K20" s="3" t="s">
-        <v>226</v>
+        <v>215</v>
       </c>
       <c r="L20" s="3" t="s">
-        <v>227</v>
+        <v>198</v>
       </c>
       <c r="M20" s="3" t="s">
-        <v>116</v>
+        <v>216</v>
       </c>
       <c r="P20" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="Q20" s="1" t="s">
-        <v>36</v>
+      <c r="Q20" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="R20" s="1" t="s">
         <v>36</v>
@@ -8169,29 +8172,29 @@
       <c r="S20" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="T20" s="2" t="s">
-        <v>35</v>
+      <c r="T20" s="1" t="s">
+        <v>36</v>
       </c>
       <c r="U20" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="V20" s="1" t="s">
-        <v>36</v>
+      <c r="V20" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="W20" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="X20" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="Y20" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="Z20" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="AA20" s="2" t="s">
-        <v>35</v>
+      <c r="X20" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="Y20" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="Z20" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AA20" s="1" t="s">
+        <v>36</v>
       </c>
       <c r="AB20" s="1" t="s">
         <v>36</v>
@@ -8202,8 +8205,8 @@
       <c r="AD20" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="AE20" s="1" t="s">
-        <v>36</v>
+      <c r="AE20" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="AF20" s="1" t="s">
         <v>36</v>
@@ -8217,10 +8220,10 @@
         <v>31</v>
       </c>
       <c r="C21" s="3">
-        <v>215</v>
+        <v>210</v>
       </c>
       <c r="D21" s="3">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="E21" s="3">
         <v>0</v>
@@ -8229,19 +8232,19 @@
         <v>70</v>
       </c>
       <c r="G21" s="3">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="J21" s="3" t="s">
-        <v>299</v>
+        <v>225</v>
       </c>
       <c r="K21" s="3" t="s">
-        <v>300</v>
+        <v>226</v>
       </c>
       <c r="L21" s="3" t="s">
-        <v>301</v>
+        <v>227</v>
       </c>
       <c r="M21" s="3" t="s">
-        <v>132</v>
+        <v>116</v>
       </c>
       <c r="P21" s="2" t="s">
         <v>35</v>
@@ -8267,14 +8270,14 @@
       <c r="W21" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="X21" s="2" t="s">
-        <v>35</v>
+      <c r="X21" s="1" t="s">
+        <v>36</v>
       </c>
       <c r="Y21" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="Z21" s="1" t="s">
-        <v>36</v>
+      <c r="Z21" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="AA21" s="2" t="s">
         <v>35</v>
@@ -8282,14 +8285,14 @@
       <c r="AB21" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="AC21" s="2" t="s">
-        <v>35</v>
+      <c r="AC21" s="1" t="s">
+        <v>36</v>
       </c>
       <c r="AD21" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="AE21" s="2" t="s">
-        <v>35</v>
+      <c r="AE21" s="1" t="s">
+        <v>36</v>
       </c>
       <c r="AF21" s="1" t="s">
         <v>36</v>
@@ -8297,16 +8300,16 @@
     </row>
     <row r="22">
       <c r="A22" s="3" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>31</v>
       </c>
       <c r="C22" s="3">
-        <v>230</v>
+        <v>215</v>
       </c>
       <c r="D22" s="3">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="E22" s="3">
         <v>0</v>
@@ -8315,19 +8318,19 @@
         <v>70</v>
       </c>
       <c r="G22" s="3">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="J22" s="3" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="K22" s="3" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="L22" s="3" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="M22" s="3" t="s">
-        <v>306</v>
+        <v>132</v>
       </c>
       <c r="P22" s="2" t="s">
         <v>35</v>
@@ -8341,17 +8344,17 @@
       <c r="S22" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="T22" s="1" t="s">
-        <v>36</v>
+      <c r="T22" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="U22" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="V22" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="W22" s="2" t="s">
-        <v>35</v>
+      <c r="V22" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="W22" s="1" t="s">
+        <v>36</v>
       </c>
       <c r="X22" s="2" t="s">
         <v>35</v>
@@ -8359,23 +8362,23 @@
       <c r="Y22" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="Z22" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="AA22" s="1" t="s">
-        <v>36</v>
+      <c r="Z22" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AA22" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="AB22" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="AC22" s="1" t="s">
-        <v>36</v>
+      <c r="AC22" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="AD22" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="AE22" s="1" t="s">
-        <v>36</v>
+      <c r="AE22" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="AF22" s="1" t="s">
         <v>36</v>
@@ -8383,16 +8386,16 @@
     </row>
     <row r="23">
       <c r="A23" s="3" t="s">
-        <v>307</v>
+        <v>303</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>31</v>
       </c>
       <c r="C23" s="3">
-        <v>280</v>
+        <v>230</v>
       </c>
       <c r="D23" s="3">
-        <v>0.45</v>
+        <v>0.3</v>
       </c>
       <c r="E23" s="3">
         <v>0</v>
@@ -8401,19 +8404,19 @@
         <v>70</v>
       </c>
       <c r="G23" s="3">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="J23" s="3" t="s">
-        <v>81</v>
+        <v>304</v>
       </c>
       <c r="K23" s="3" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="L23" s="3" t="s">
-        <v>83</v>
+        <v>306</v>
       </c>
       <c r="M23" s="3" t="s">
-        <v>116</v>
+        <v>307</v>
       </c>
       <c r="P23" s="2" t="s">
         <v>35</v>
@@ -8439,11 +8442,11 @@
       <c r="W23" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="X23" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="Y23" s="2" t="s">
-        <v>35</v>
+      <c r="X23" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="Y23" s="1" t="s">
+        <v>36</v>
       </c>
       <c r="Z23" s="2" t="s">
         <v>35</v>
@@ -8451,8 +8454,8 @@
       <c r="AA23" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="AB23" s="2" t="s">
-        <v>35</v>
+      <c r="AB23" s="1" t="s">
+        <v>36</v>
       </c>
       <c r="AC23" s="1" t="s">
         <v>36</v>
@@ -8463,43 +8466,43 @@
       <c r="AE23" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="AF23" s="2" t="s">
-        <v>35</v>
+      <c r="AF23" s="1" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>31</v>
       </c>
       <c r="C24" s="3">
-        <v>140</v>
+        <v>280</v>
       </c>
       <c r="D24" s="3">
-        <v>0.25</v>
+        <v>0.45</v>
       </c>
       <c r="E24" s="3">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="F24" s="3">
-        <v>180</v>
+        <v>70</v>
       </c>
       <c r="G24" s="3">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="J24" s="3" t="s">
-        <v>310</v>
+        <v>81</v>
       </c>
       <c r="K24" s="3" t="s">
-        <v>278</v>
+        <v>309</v>
       </c>
       <c r="L24" s="3" t="s">
-        <v>311</v>
+        <v>83</v>
       </c>
       <c r="M24" s="3" t="s">
-        <v>312</v>
+        <v>116</v>
       </c>
       <c r="P24" s="2" t="s">
         <v>35</v>
@@ -8516,29 +8519,29 @@
       <c r="T24" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="U24" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="V24" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="W24" s="1" t="s">
-        <v>36</v>
+      <c r="U24" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="V24" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="W24" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="X24" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="Y24" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="Z24" s="1" t="s">
-        <v>36</v>
+      <c r="Y24" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="Z24" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="AA24" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="AB24" s="1" t="s">
-        <v>36</v>
+      <c r="AB24" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="AC24" s="1" t="s">
         <v>36</v>
@@ -8549,19 +8552,19 @@
       <c r="AE24" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="AF24" s="1" t="s">
-        <v>36</v>
+      <c r="AF24" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>31</v>
       </c>
       <c r="C25" s="3">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="D25" s="3">
         <v>0.25</v>
@@ -8576,13 +8579,16 @@
         <v>45</v>
       </c>
       <c r="J25" s="3" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
       <c r="K25" s="3" t="s">
-        <v>234</v>
+        <v>278</v>
       </c>
       <c r="L25" s="3" t="s">
-        <v>111</v>
+        <v>312</v>
+      </c>
+      <c r="M25" s="3" t="s">
+        <v>313</v>
       </c>
       <c r="P25" s="2" t="s">
         <v>35</v>
@@ -8638,13 +8644,13 @@
     </row>
     <row r="26">
       <c r="A26" s="3" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="B26" s="3" t="s">
         <v>31</v>
       </c>
       <c r="C26" s="3">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="D26" s="3">
         <v>0.25</v>
@@ -8659,16 +8665,13 @@
         <v>45</v>
       </c>
       <c r="J26" s="3" t="s">
-        <v>146</v>
+        <v>315</v>
       </c>
       <c r="K26" s="3" t="s">
-        <v>145</v>
+        <v>234</v>
       </c>
       <c r="L26" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="M26" s="3" t="s">
-        <v>316</v>
+        <v>111</v>
       </c>
       <c r="P26" s="2" t="s">
         <v>35</v>
@@ -8724,13 +8727,13 @@
     </row>
     <row r="27">
       <c r="A27" s="3" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="B27" s="3" t="s">
         <v>31</v>
       </c>
       <c r="C27" s="3">
-        <v>150</v>
+        <v>140</v>
       </c>
       <c r="D27" s="3">
         <v>0.25</v>
@@ -8745,19 +8748,16 @@
         <v>45</v>
       </c>
       <c r="J27" s="3" t="s">
-        <v>220</v>
+        <v>146</v>
       </c>
       <c r="K27" s="3" t="s">
-        <v>290</v>
+        <v>145</v>
       </c>
       <c r="L27" s="3" t="s">
-        <v>206</v>
+        <v>55</v>
       </c>
       <c r="M27" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="N27" s="3" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="P27" s="2" t="s">
         <v>35</v>
@@ -8813,13 +8813,13 @@
     </row>
     <row r="28">
       <c r="A28" s="3" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="B28" s="3" t="s">
         <v>31</v>
       </c>
       <c r="C28" s="3">
-        <v>140</v>
+        <v>150</v>
       </c>
       <c r="D28" s="3">
         <v>0.25</v>
@@ -8834,66 +8834,155 @@
         <v>45</v>
       </c>
       <c r="J28" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="K28" s="3" t="s">
+        <v>291</v>
+      </c>
+      <c r="L28" s="3" t="s">
+        <v>206</v>
+      </c>
+      <c r="M28" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="N28" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="P28" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q28" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="R28" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="S28" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="T28" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="U28" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="V28" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="W28" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="X28" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="Y28" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="Z28" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AA28" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AB28" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AC28" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AD28" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="AE28" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AF28" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="s">
         <v>320</v>
       </c>
-      <c r="K28" s="3" t="s">
+      <c r="B29" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C29" s="3">
+        <v>140</v>
+      </c>
+      <c r="D29" s="3">
+        <v>0.25</v>
+      </c>
+      <c r="E29" s="3">
+        <v>80</v>
+      </c>
+      <c r="F29" s="3">
+        <v>180</v>
+      </c>
+      <c r="G29" s="3">
+        <v>45</v>
+      </c>
+      <c r="J29" s="3" t="s">
+        <v>321</v>
+      </c>
+      <c r="K29" s="3" t="s">
         <v>246</v>
       </c>
-      <c r="L28" s="3" t="s">
+      <c r="L29" s="3" t="s">
         <v>227</v>
       </c>
-      <c r="M28" s="3" t="s">
-        <v>321</v>
-      </c>
-      <c r="P28" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="Q28" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="R28" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="S28" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="T28" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="U28" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="V28" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="W28" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="X28" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="Y28" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="Z28" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="AA28" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="AB28" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="AC28" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="AD28" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="AE28" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="AF28" s="1" t="s">
+      <c r="M29" s="3" t="s">
+        <v>322</v>
+      </c>
+      <c r="P29" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q29" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="R29" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="S29" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="T29" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="U29" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="V29" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="W29" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="X29" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="Y29" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="Z29" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AA29" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AB29" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AC29" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AD29" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="AE29" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AF29" s="1" t="s">
         <v>36</v>
       </c>
     </row>
@@ -9002,16 +9091,16 @@
         <v>19</v>
       </c>
       <c r="U1" s="4" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="V1" s="4" t="s">
         <v>21</v>
       </c>
       <c r="W1" s="4" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="X1" s="4" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="Y1" s="4" t="s">
         <v>26</v>
@@ -9019,7 +9108,7 @@
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>31</v>
@@ -9040,16 +9129,16 @@
         <v>35</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="K2" s="3" t="s">
         <v>91</v>
       </c>
       <c r="L2" s="3" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="M2" s="3" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="P2" s="2" t="s">
         <v>35</v>
@@ -9084,7 +9173,7 @@
     </row>
     <row r="3">
       <c r="A3" s="3" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>31</v>
@@ -9105,13 +9194,13 @@
         <v>40</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="P3" s="2" t="s">
         <v>35</v>
@@ -9146,7 +9235,7 @@
     </row>
     <row r="4">
       <c r="A4" s="3" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>99</v>
@@ -9170,16 +9259,16 @@
         <v>8</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="M4" s="3" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="N4" s="3" t="s">
         <v>214</v>
@@ -9217,7 +9306,7 @@
     </row>
     <row r="5">
       <c r="A5" s="3" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>31</v>
@@ -9238,16 +9327,16 @@
         <v>35</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="L5" s="3" t="s">
         <v>109</v>
       </c>
       <c r="M5" s="3" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="P5" s="2" t="s">
         <v>35</v>
@@ -9282,7 +9371,7 @@
     </row>
     <row r="6">
       <c r="A6" s="3" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>31</v>
@@ -9347,7 +9436,7 @@
     </row>
     <row r="7">
       <c r="A7" s="3" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>31</v>
@@ -9368,16 +9457,16 @@
         <v>30</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="K7" s="3" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="L7" s="3" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="M7" s="3" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="P7" s="1" t="s">
         <v>36</v>
@@ -9412,7 +9501,7 @@
     </row>
     <row r="8">
       <c r="A8" s="3" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>38</v>
@@ -9436,16 +9525,16 @@
         <v>7</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="K8" s="3" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="L8" s="3" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="M8" s="3" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="P8" s="1" t="s">
         <v>36</v>
@@ -9480,7 +9569,7 @@
     </row>
     <row r="9">
       <c r="A9" s="3" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>31</v>
@@ -9501,16 +9590,16 @@
         <v>45</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="K9" s="3" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="L9" s="3" t="s">
         <v>127</v>
       </c>
       <c r="M9" s="3" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="N9" s="3" t="s">
         <v>129</v>
@@ -9548,7 +9637,7 @@
     </row>
     <row r="10">
       <c r="A10" s="3" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>38</v>
@@ -9578,7 +9667,7 @@
         <v>272</v>
       </c>
       <c r="L10" s="3" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="M10" s="3" t="s">
         <v>133</v>
@@ -9616,7 +9705,7 @@
     </row>
     <row r="11">
       <c r="A11" s="3" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>99</v>
@@ -9640,13 +9729,13 @@
         <v>9</v>
       </c>
       <c r="J11" s="3" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="K11" s="3" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="L11" s="3" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="P11" s="2" t="s">
         <v>35</v>
@@ -9681,7 +9770,7 @@
     </row>
     <row r="12">
       <c r="A12" s="3" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>38</v>
@@ -9708,16 +9797,16 @@
         <v>139</v>
       </c>
       <c r="K12" s="3" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="L12" s="3" t="s">
         <v>204</v>
       </c>
       <c r="M12" s="3" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="N12" s="3" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="P12" s="2" t="s">
         <v>35</v>
@@ -9752,7 +9841,7 @@
     </row>
     <row r="13">
       <c r="A13" s="3" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>31</v>
@@ -9820,7 +9909,7 @@
     </row>
     <row r="14">
       <c r="A14" s="3" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>31</v>
@@ -9841,13 +9930,13 @@
         <v>50</v>
       </c>
       <c r="J14" s="3" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="K14" s="3" t="s">
         <v>63</v>
       </c>
       <c r="L14" s="3" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="M14" s="3" t="s">
         <v>65</v>
@@ -9888,7 +9977,7 @@
     </row>
     <row r="15">
       <c r="A15" s="3" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>31</v>
@@ -9953,7 +10042,7 @@
     </row>
     <row r="16">
       <c r="A16" s="3" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>31</v>
@@ -9974,7 +10063,7 @@
         <v>35</v>
       </c>
       <c r="J16" s="3" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="K16" s="3" t="s">
         <v>173</v>
@@ -9983,10 +10072,10 @@
         <v>174</v>
       </c>
       <c r="M16" s="3" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="N16" s="3" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="P16" s="2" t="s">
         <v>35</v>
@@ -10021,7 +10110,7 @@
     </row>
     <row r="17">
       <c r="A17" s="3" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>31</v>
@@ -10051,7 +10140,7 @@
         <v>70</v>
       </c>
       <c r="M17" s="3" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="P17" s="2" t="s">
         <v>35</v>
@@ -10086,7 +10175,7 @@
     </row>
     <row r="18">
       <c r="A18" s="3" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>31</v>
@@ -10107,7 +10196,7 @@
         <v>40</v>
       </c>
       <c r="J18" s="3" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="K18" s="3" t="s">
         <v>178</v>
@@ -10116,7 +10205,7 @@
         <v>179</v>
       </c>
       <c r="M18" s="3" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="P18" s="1" t="s">
         <v>36</v>
@@ -10151,7 +10240,7 @@
     </row>
     <row r="19">
       <c r="A19" s="3" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>31</v>
@@ -10172,16 +10261,16 @@
         <v>35</v>
       </c>
       <c r="J19" s="3" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="K19" s="3" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="L19" s="3" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="M19" s="3" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="P19" s="1" t="s">
         <v>36</v>
@@ -10216,7 +10305,7 @@
     </row>
     <row r="20">
       <c r="A20" s="3" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>31</v>
@@ -10237,16 +10326,16 @@
         <v>45</v>
       </c>
       <c r="J20" s="3" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="K20" s="3" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="L20" s="3" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="M20" s="3" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="P20" s="1" t="s">
         <v>36</v>
@@ -10281,7 +10370,7 @@
     </row>
     <row r="21">
       <c r="A21" s="3" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>31</v>
@@ -10311,7 +10400,7 @@
         <v>194</v>
       </c>
       <c r="M21" s="3" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="P21" s="1" t="s">
         <v>36</v>
@@ -10346,7 +10435,7 @@
     </row>
     <row r="22">
       <c r="A22" s="3" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>31</v>
@@ -10367,16 +10456,16 @@
         <v>30</v>
       </c>
       <c r="J22" s="3" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="K22" s="3" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="L22" s="3" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="M22" s="3" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="P22" s="1" t="s">
         <v>36</v>
@@ -10411,7 +10500,7 @@
     </row>
     <row r="23">
       <c r="A23" s="3" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>38</v>
@@ -10447,7 +10536,7 @@
         <v>79</v>
       </c>
       <c r="N23" s="3" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="P23" s="2" t="s">
         <v>35</v>
@@ -10482,7 +10571,7 @@
     </row>
     <row r="24">
       <c r="A24" s="3" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>31</v>
@@ -10503,13 +10592,13 @@
         <v>20</v>
       </c>
       <c r="J24" s="3" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="K24" s="3" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="L24" s="3" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="P24" s="2" t="s">
         <v>35</v>
@@ -10544,7 +10633,7 @@
     </row>
     <row r="25">
       <c r="A25" s="3" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>31</v>
@@ -10568,13 +10657,13 @@
         <v>206</v>
       </c>
       <c r="K25" s="3" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="L25" s="3" t="s">
         <v>269</v>
       </c>
       <c r="M25" s="3" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="P25" s="2" t="s">
         <v>35</v>
@@ -10609,7 +10698,7 @@
     </row>
     <row r="26">
       <c r="A26" s="3" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="B26" s="3" t="s">
         <v>31</v>
@@ -10630,13 +10719,13 @@
         <v>35</v>
       </c>
       <c r="J26" s="3" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="K26" s="3" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="L26" s="3" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="P26" s="1" t="s">
         <v>36</v>
@@ -10671,7 +10760,7 @@
     </row>
     <row r="27">
       <c r="A27" s="3" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="B27" s="3" t="s">
         <v>31</v>
@@ -10692,16 +10781,16 @@
         <v>35</v>
       </c>
       <c r="J27" s="3" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="K27" s="3" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="L27" s="3" t="s">
         <v>227</v>
       </c>
       <c r="M27" s="3" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="P27" s="1" t="s">
         <v>36</v>
@@ -10736,7 +10825,7 @@
     </row>
     <row r="28">
       <c r="A28" s="3" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="B28" s="3" t="s">
         <v>38</v>
@@ -10895,16 +10984,16 @@
         <v>11</v>
       </c>
       <c r="Q1" s="4" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="R1" s="4" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="S1" s="4" t="s">
         <v>17</v>
       </c>
       <c r="T1" s="4" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="U1" s="4" t="s">
         <v>19</v>
@@ -10921,7 +11010,7 @@
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>38</v>
@@ -10945,7 +11034,7 @@
         <v>4</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="P2" s="2" t="s">
         <v>35</v>
@@ -10977,7 +11066,7 @@
     </row>
     <row r="3">
       <c r="A3" s="3" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>31</v>
@@ -10998,10 +11087,10 @@
         <v>39</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="L3" s="3" t="s">
         <v>92</v>
@@ -11036,7 +11125,7 @@
     </row>
     <row r="4">
       <c r="A4" s="3" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>38</v>
@@ -11060,13 +11149,13 @@
         <v>9</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="M4" s="3" t="s">
         <v>97</v>
@@ -11101,7 +11190,7 @@
     </row>
     <row r="5">
       <c r="A5" s="3" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>99</v>
@@ -11125,13 +11214,13 @@
         <v>12</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="L5" s="3" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="M5" s="3" t="s">
         <v>214</v>
@@ -11166,7 +11255,7 @@
     </row>
     <row r="6">
       <c r="A6" s="3" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>31</v>
@@ -11187,10 +11276,10 @@
         <v>45</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="K6" s="3" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="L6" s="3" t="s">
         <v>111</v>
@@ -11225,7 +11314,7 @@
     </row>
     <row r="7">
       <c r="A7" s="3" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>31</v>
@@ -11255,7 +11344,7 @@
         <v>34</v>
       </c>
       <c r="M7" s="3" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="P7" s="1" t="s">
         <v>36</v>
@@ -11287,7 +11376,7 @@
     </row>
     <row r="8">
       <c r="A8" s="3" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>31</v>
@@ -11308,16 +11397,16 @@
         <v>45</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="K8" s="3" t="s">
         <v>116</v>
       </c>
       <c r="L8" s="3" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="M8" s="3" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="P8" s="1" t="s">
         <v>36</v>
@@ -11349,7 +11438,7 @@
     </row>
     <row r="9">
       <c r="A9" s="3" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>38</v>
@@ -11373,16 +11462,16 @@
         <v>8</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="K9" s="3" t="s">
         <v>40</v>
       </c>
       <c r="L9" s="3" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="M9" s="3" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="P9" s="1" t="s">
         <v>36</v>
@@ -11414,7 +11503,7 @@
     </row>
     <row r="10">
       <c r="A10" s="3" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>31</v>
@@ -11435,13 +11524,13 @@
         <v>45</v>
       </c>
       <c r="J10" s="3" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="K10" s="3" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="L10" s="3" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="M10" s="3" t="s">
         <v>123</v>
@@ -11476,7 +11565,7 @@
     </row>
     <row r="11">
       <c r="A11" s="3" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>31</v>
@@ -11497,16 +11586,16 @@
         <v>45</v>
       </c>
       <c r="J11" s="3" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="K11" s="3" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="L11" s="3" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="M11" s="3" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="N11" s="3" t="s">
         <v>129</v>
@@ -11541,7 +11630,7 @@
     </row>
     <row r="12">
       <c r="A12" s="3" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>31</v>
@@ -11562,10 +11651,10 @@
         <v>37</v>
       </c>
       <c r="J12" s="3" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="K12" s="3" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="L12" s="3" t="s">
         <v>49</v>
@@ -11603,7 +11692,7 @@
     </row>
     <row r="13">
       <c r="A13" s="3" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>31</v>
@@ -11665,7 +11754,7 @@
     </row>
     <row r="14">
       <c r="A14" s="3" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>99</v>
@@ -11692,10 +11781,10 @@
         <v>275</v>
       </c>
       <c r="K14" s="3" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="L14" s="3" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="P14" s="2" t="s">
         <v>35</v>
@@ -11727,7 +11816,7 @@
     </row>
     <row r="15">
       <c r="A15" s="3" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>38</v>
@@ -11751,16 +11840,16 @@
         <v>9</v>
       </c>
       <c r="J15" s="3" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="K15" s="3" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="L15" s="3" t="s">
         <v>141</v>
       </c>
       <c r="M15" s="3" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="P15" s="2" t="s">
         <v>35</v>
@@ -11792,7 +11881,7 @@
     </row>
     <row r="16">
       <c r="A16" s="3" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>31</v>
@@ -11819,7 +11908,7 @@
         <v>53</v>
       </c>
       <c r="L16" s="3" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="M16" s="3" t="s">
         <v>55</v>
@@ -11857,7 +11946,7 @@
     </row>
     <row r="17">
       <c r="A17" s="3" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>31</v>
@@ -11878,13 +11967,13 @@
         <v>40</v>
       </c>
       <c r="J17" s="3" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="K17" s="3" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="L17" s="3" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="M17" s="3" t="s">
         <v>151</v>
@@ -11919,7 +12008,7 @@
     </row>
     <row r="18">
       <c r="A18" s="3" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>31</v>
@@ -11940,16 +12029,16 @@
         <v>41</v>
       </c>
       <c r="J18" s="3" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="K18" s="3" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="L18" s="3" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="M18" s="3" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="N18" s="3" t="s">
         <v>160</v>
@@ -11984,7 +12073,7 @@
     </row>
     <row r="19">
       <c r="A19" s="3" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>31</v>
@@ -12005,16 +12094,16 @@
         <v>39</v>
       </c>
       <c r="J19" s="3" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="K19" s="3" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="L19" s="3" t="s">
         <v>165</v>
       </c>
       <c r="M19" s="3" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="N19" s="3" t="s">
         <v>66</v>
@@ -12049,7 +12138,7 @@
     </row>
     <row r="20">
       <c r="A20" s="3" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>31</v>
@@ -12070,13 +12159,13 @@
         <v>45</v>
       </c>
       <c r="J20" s="3" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="K20" s="3" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="L20" s="3" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="M20" s="3" t="s">
         <v>170</v>
@@ -12111,7 +12200,7 @@
     </row>
     <row r="21">
       <c r="A21" s="3" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>31</v>
@@ -12132,13 +12221,13 @@
         <v>41</v>
       </c>
       <c r="J21" s="3" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="K21" s="3" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="L21" s="3" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="P21" s="2" t="s">
         <v>35</v>
@@ -12170,7 +12259,7 @@
     </row>
     <row r="22">
       <c r="A22" s="3" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>31</v>
@@ -12197,10 +12286,10 @@
         <v>69</v>
       </c>
       <c r="L22" s="3" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="M22" s="3" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="P22" s="2" t="s">
         <v>35</v>
@@ -12232,7 +12321,7 @@
     </row>
     <row r="23">
       <c r="A23" s="3" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>31</v>
@@ -12253,13 +12342,13 @@
         <v>45</v>
       </c>
       <c r="J23" s="3" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="K23" s="3" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="L23" s="3" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="P23" s="2" t="s">
         <v>35</v>
@@ -12291,7 +12380,7 @@
     </row>
     <row r="24">
       <c r="A24" s="3" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>31</v>
@@ -12312,7 +12401,7 @@
         <v>32</v>
       </c>
       <c r="J24" s="3" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="P24" s="1" t="s">
         <v>36</v>
@@ -12344,7 +12433,7 @@
     </row>
     <row r="25">
       <c r="A25" s="3" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>31</v>
@@ -12365,13 +12454,13 @@
         <v>31</v>
       </c>
       <c r="J25" s="3" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="K25" s="3" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="L25" s="3" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="M25" s="3" t="s">
         <v>186</v>
@@ -12406,7 +12495,7 @@
     </row>
     <row r="26">
       <c r="A26" s="3" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="B26" s="3" t="s">
         <v>31</v>
@@ -12465,7 +12554,7 @@
     </row>
     <row r="27">
       <c r="A27" s="3" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="B27" s="3" t="s">
         <v>31</v>
@@ -12486,13 +12575,13 @@
         <v>45</v>
       </c>
       <c r="J27" s="3" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="K27" s="3" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="L27" s="3" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="P27" s="1" t="s">
         <v>36</v>
@@ -12524,7 +12613,7 @@
     </row>
     <row r="28">
       <c r="A28" s="3" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="B28" s="3" t="s">
         <v>31</v>
@@ -12548,10 +12637,10 @@
         <v>192</v>
       </c>
       <c r="K28" s="3" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="L28" s="3" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="P28" s="2" t="s">
         <v>35</v>
@@ -12583,7 +12672,7 @@
     </row>
     <row r="29">
       <c r="A29" s="3" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="B29" s="3" t="s">
         <v>31</v>
@@ -12604,13 +12693,13 @@
         <v>50</v>
       </c>
       <c r="J29" s="3" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="K29" s="3" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="L29" s="3" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="M29" s="3" t="s">
         <v>204</v>
@@ -12645,7 +12734,7 @@
     </row>
     <row r="30">
       <c r="A30" s="3" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="B30" s="3" t="s">
         <v>38</v>
@@ -12675,10 +12764,10 @@
         <v>77</v>
       </c>
       <c r="L30" s="3" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="M30" s="3" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="P30" s="2" t="s">
         <v>35</v>
@@ -12710,7 +12799,7 @@
     </row>
     <row r="31">
       <c r="A31" s="3" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="B31" s="3" t="s">
         <v>31</v>
@@ -12731,13 +12820,13 @@
         <v>25</v>
       </c>
       <c r="J31" s="3" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="K31" s="3" t="s">
         <v>82</v>
       </c>
       <c r="L31" s="3" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="P31" s="2" t="s">
         <v>35</v>
@@ -12769,7 +12858,7 @@
     </row>
     <row r="32">
       <c r="A32" s="3" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="B32" s="3" t="s">
         <v>31</v>
@@ -12793,10 +12882,10 @@
         <v>268</v>
       </c>
       <c r="K32" s="3" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="L32" s="3" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="P32" s="2" t="s">
         <v>35</v>
@@ -12828,7 +12917,7 @@
     </row>
     <row r="33">
       <c r="A33" s="3" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="B33" s="3" t="s">
         <v>31</v>
@@ -12849,13 +12938,13 @@
         <v>45</v>
       </c>
       <c r="J33" s="3" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="K33" s="3" t="s">
         <v>211</v>
       </c>
       <c r="L33" s="3" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="P33" s="1" t="s">
         <v>36</v>
@@ -12887,7 +12976,7 @@
     </row>
     <row r="34">
       <c r="A34" s="3" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="B34" s="3" t="s">
         <v>31</v>
@@ -12908,13 +12997,13 @@
         <v>50</v>
       </c>
       <c r="J34" s="3" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="K34" s="3" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="L34" s="3" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="P34" s="1" t="s">
         <v>36</v>
@@ -12946,7 +13035,7 @@
     </row>
     <row r="35">
       <c r="A35" s="3" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="B35" s="3" t="s">
         <v>31</v>
@@ -12967,7 +13056,7 @@
         <v>17</v>
       </c>
       <c r="J35" s="3" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="P35" s="2" t="s">
         <v>35</v>
@@ -12999,7 +13088,7 @@
     </row>
     <row r="36">
       <c r="A36" s="3" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="B36" s="3" t="s">
         <v>31</v>
@@ -13020,10 +13109,10 @@
         <v>45</v>
       </c>
       <c r="J36" s="3" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="K36" s="3" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="L36" s="3" t="s">
         <v>227</v>
@@ -13058,7 +13147,7 @@
     </row>
     <row r="37">
       <c r="A37" s="3" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="B37" s="3" t="s">
         <v>38</v>
@@ -13220,7 +13309,7 @@
         <v>16</v>
       </c>
       <c r="S1" s="4" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="T1" s="4" t="s">
         <v>26</v>
@@ -13231,7 +13320,7 @@
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>38</v>
@@ -13255,16 +13344,16 @@
         <v>6</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="L2" s="3" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="M2" s="3" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="P2" s="1" t="s">
         <v>36</v>
@@ -13287,7 +13376,7 @@
     </row>
     <row r="3">
       <c r="A3" s="3" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>31</v>
@@ -13308,13 +13397,13 @@
         <v>20</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="P3" s="1" t="s">
         <v>36</v>

</xml_diff>

<commit_message>
remove diamond/graphite from sedimentary
</commit_message>
<xml_diff>
--- a/OresToFieldGuide/data/sheet.xlsx
+++ b/OresToFieldGuide/data/sheet.xlsx
@@ -4016,17 +4016,17 @@
       <c r="Q25" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="R25" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="S25" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="T25" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="U25" s="1" t="s">
-        <v>36</v>
+      <c r="R25" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="S25" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="T25" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="U25" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="V25" s="1" t="s">
         <v>36</v>
@@ -4034,8 +4034,8 @@
       <c r="W25" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="X25" s="1" t="s">
-        <v>36</v>
+      <c r="X25" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="Y25" s="1" t="s">
         <v>36</v>
@@ -4046,8 +4046,8 @@
       <c r="AA25" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="AB25" s="1" t="s">
-        <v>36</v>
+      <c r="AB25" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="AC25" s="1" t="s">
         <v>36</v>
@@ -4064,8 +4064,8 @@
       <c r="AG25" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="AH25" s="1" t="s">
-        <v>36</v>
+      <c r="AH25" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="AI25" s="1" t="s">
         <v>36</v>

</xml_diff>

<commit_message>
add new ore blocks
</commit_message>
<xml_diff>
--- a/OresToFieldGuide/data/sheet.xlsx
+++ b/OresToFieldGuide/data/sheet.xlsx
@@ -1705,7 +1705,10 @@
     <col min="43" max="43" width="9.140625" customWidth="1" style="3"/>
     <col min="44" max="44" width="9.140625" customWidth="1" style="3"/>
     <col min="45" max="45" width="9.140625" customWidth="1" style="3"/>
-    <col min="46" max="16384" width="9.140625" customWidth="1" style="3"/>
+    <col min="46" max="46" width="9.140625" customWidth="1" style="3"/>
+    <col min="47" max="47" width="9.140625" customWidth="1" style="3"/>
+    <col min="48" max="48" width="9.140625" customWidth="1" style="3"/>
+    <col min="49" max="16384" width="9.140625" customWidth="1" style="3"/>
   </cols>
   <sheetData>
     <row r="1" s="4" customFormat="1">
@@ -6572,7 +6575,10 @@
     <col min="43" max="43" width="9.140625" customWidth="1" style="3"/>
     <col min="44" max="44" width="9.140625" customWidth="1" style="3"/>
     <col min="45" max="45" width="9.140625" customWidth="1" style="3"/>
-    <col min="46" max="16384" width="9.140625" customWidth="1" style="3"/>
+    <col min="46" max="46" width="9.140625" customWidth="1" style="3"/>
+    <col min="47" max="47" width="9.140625" customWidth="1" style="3"/>
+    <col min="48" max="48" width="9.140625" customWidth="1" style="3"/>
+    <col min="49" max="16384" width="9.140625" customWidth="1" style="3"/>
   </cols>
   <sheetData>
     <row r="1" s="4" customFormat="1">
@@ -9211,7 +9217,10 @@
     <col min="43" max="43" width="9.140625" customWidth="1" style="3"/>
     <col min="44" max="44" width="9.140625" customWidth="1" style="3"/>
     <col min="45" max="45" width="9.140625" customWidth="1" style="3"/>
-    <col min="46" max="16384" width="9.140625" customWidth="1" style="3"/>
+    <col min="46" max="46" width="9.140625" customWidth="1" style="3"/>
+    <col min="47" max="47" width="9.140625" customWidth="1" style="3"/>
+    <col min="48" max="48" width="9.140625" customWidth="1" style="3"/>
+    <col min="49" max="16384" width="9.140625" customWidth="1" style="3"/>
   </cols>
   <sheetData>
     <row r="1" s="4" customFormat="1">
@@ -11116,7 +11125,10 @@
     <col min="43" max="43" width="9.140625" customWidth="1" style="3"/>
     <col min="44" max="44" width="9.140625" customWidth="1" style="3"/>
     <col min="45" max="45" width="9.140625" customWidth="1" style="3"/>
-    <col min="46" max="16384" width="9.140625" customWidth="1" style="3"/>
+    <col min="46" max="46" width="9.140625" customWidth="1" style="3"/>
+    <col min="47" max="47" width="9.140625" customWidth="1" style="3"/>
+    <col min="48" max="48" width="9.140625" customWidth="1" style="3"/>
+    <col min="49" max="16384" width="9.140625" customWidth="1" style="3"/>
   </cols>
   <sheetData>
     <row r="1" s="4" customFormat="1">
@@ -13382,7 +13394,10 @@
     <col min="43" max="43" width="9.140625" customWidth="1" style="3"/>
     <col min="44" max="44" width="9.140625" customWidth="1" style="3"/>
     <col min="45" max="45" width="9.140625" customWidth="1" style="3"/>
-    <col min="46" max="16384" width="9.140625" customWidth="1" style="3"/>
+    <col min="46" max="46" width="9.140625" customWidth="1" style="3"/>
+    <col min="47" max="47" width="9.140625" customWidth="1" style="3"/>
+    <col min="48" max="48" width="9.140625" customWidth="1" style="3"/>
+    <col min="49" max="16384" width="9.140625" customWidth="1" style="3"/>
   </cols>
   <sheetData>
     <row r="1" s="4" customFormat="1">

</xml_diff>

<commit_message>
tweaked ores a little
</commit_message>
<xml_diff>
--- a/OresToFieldGuide/data/sheet.xlsx
+++ b/OresToFieldGuide/data/sheet.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="525" uniqueCount="525">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="523" uniqueCount="523">
   <si>
     <t>Vein ID</t>
   </si>
@@ -510,13 +510,10 @@
     <t>normal_magnetite</t>
   </si>
   <si>
-    <t>magnetite: 70 [1]</t>
-  </si>
-  <si>
-    <t>vanadium_magnetite: 25</t>
-  </si>
-  <si>
-    <t>gold: 10</t>
+    <t>magnetite: 60 [1]</t>
+  </si>
+  <si>
+    <t>vanadium_magnetite: 30</t>
   </si>
   <si>
     <t>chromite: 5</t>
@@ -732,10 +729,7 @@
     <t>chalcopyrite: 55</t>
   </si>
   <si>
-    <t>zeolite: 15</t>
-  </si>
-  <si>
-    <t>cassiterite: 5</t>
+    <t>zeolite: 20</t>
   </si>
   <si>
     <t>realgar: 15</t>
@@ -3894,7 +3888,7 @@
         <v>38</v>
       </c>
       <c r="C24" s="3">
-        <v>170</v>
+        <v>210</v>
       </c>
       <c r="D24" s="3">
         <v>0.4</v>
@@ -4589,10 +4583,10 @@
         <v>165</v>
       </c>
       <c r="L31" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="M31" s="3" t="s">
         <v>166</v>
-      </c>
-      <c r="M31" s="3" t="s">
-        <v>167</v>
       </c>
       <c r="P31" s="2" t="s">
         <v>35</v>
@@ -4657,7 +4651,7 @@
     </row>
     <row r="32">
       <c r="A32" s="3" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B32" s="3" t="s">
         <v>31</v>
@@ -4678,16 +4672,16 @@
         <v>30</v>
       </c>
       <c r="J32" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="K32" s="3" t="s">
         <v>169</v>
       </c>
-      <c r="K32" s="3" t="s">
+      <c r="L32" s="3" t="s">
         <v>170</v>
       </c>
-      <c r="L32" s="3" t="s">
+      <c r="M32" s="3" t="s">
         <v>171</v>
-      </c>
-      <c r="M32" s="3" t="s">
-        <v>172</v>
       </c>
       <c r="P32" s="1" t="s">
         <v>36</v>
@@ -4752,37 +4746,37 @@
     </row>
     <row r="33">
       <c r="A33" s="3" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B33" s="3" t="s">
         <v>31</v>
       </c>
       <c r="C33" s="3">
-        <v>190</v>
+        <v>230</v>
       </c>
       <c r="D33" s="3">
         <v>0.25</v>
       </c>
       <c r="E33" s="3">
-        <v>0</v>
+        <v>-32</v>
       </c>
       <c r="F33" s="3">
-        <v>210</v>
+        <v>140</v>
       </c>
       <c r="G33" s="3">
         <v>36</v>
       </c>
       <c r="J33" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="K33" s="3" t="s">
         <v>174</v>
       </c>
-      <c r="K33" s="3" t="s">
+      <c r="L33" s="3" t="s">
         <v>175</v>
       </c>
-      <c r="L33" s="3" t="s">
+      <c r="M33" s="3" t="s">
         <v>176</v>
-      </c>
-      <c r="M33" s="3" t="s">
-        <v>177</v>
       </c>
       <c r="P33" s="2" t="s">
         <v>35</v>
@@ -4847,7 +4841,7 @@
     </row>
     <row r="34">
       <c r="A34" s="3" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B34" s="3" t="s">
         <v>31</v>
@@ -4868,13 +4862,13 @@
         <v>35</v>
       </c>
       <c r="J34" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="K34" s="3" t="s">
         <v>179</v>
       </c>
-      <c r="K34" s="3" t="s">
+      <c r="L34" s="3" t="s">
         <v>180</v>
-      </c>
-      <c r="L34" s="3" t="s">
-        <v>181</v>
       </c>
       <c r="P34" s="2" t="s">
         <v>35</v>
@@ -4939,7 +4933,7 @@
     </row>
     <row r="35">
       <c r="A35" s="3" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B35" s="3" t="s">
         <v>31</v>
@@ -5025,7 +5019,7 @@
     </row>
     <row r="36">
       <c r="A36" s="3" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B36" s="3" t="s">
         <v>31</v>
@@ -5046,16 +5040,16 @@
         <v>26</v>
       </c>
       <c r="J36" s="3" t="s">
+        <v>183</v>
+      </c>
+      <c r="K36" s="3" t="s">
         <v>184</v>
       </c>
-      <c r="K36" s="3" t="s">
+      <c r="L36" s="3" t="s">
         <v>185</v>
       </c>
-      <c r="L36" s="3" t="s">
+      <c r="M36" s="3" t="s">
         <v>186</v>
-      </c>
-      <c r="M36" s="3" t="s">
-        <v>187</v>
       </c>
       <c r="P36" s="1" t="s">
         <v>36</v>
@@ -5120,7 +5114,7 @@
     </row>
     <row r="37">
       <c r="A37" s="3" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B37" s="3" t="s">
         <v>31</v>
@@ -5141,13 +5135,13 @@
         <v>40</v>
       </c>
       <c r="J37" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="K37" s="3" t="s">
         <v>189</v>
       </c>
-      <c r="K37" s="3" t="s">
+      <c r="L37" s="3" t="s">
         <v>190</v>
-      </c>
-      <c r="L37" s="3" t="s">
-        <v>191</v>
       </c>
       <c r="P37" s="2" t="s">
         <v>35</v>
@@ -5212,7 +5206,7 @@
     </row>
     <row r="38">
       <c r="A38" s="3" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B38" s="3" t="s">
         <v>31</v>
@@ -5233,13 +5227,13 @@
         <v>40</v>
       </c>
       <c r="J38" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="K38" s="3" t="s">
         <v>193</v>
       </c>
-      <c r="K38" s="3" t="s">
+      <c r="L38" s="3" t="s">
         <v>194</v>
-      </c>
-      <c r="L38" s="3" t="s">
-        <v>195</v>
       </c>
       <c r="P38" s="2" t="s">
         <v>35</v>
@@ -5304,7 +5298,7 @@
     </row>
     <row r="39">
       <c r="A39" s="3" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B39" s="3" t="s">
         <v>38</v>
@@ -5328,16 +5322,16 @@
         <v>4</v>
       </c>
       <c r="J39" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="K39" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="K39" s="3" t="s">
+      <c r="L39" s="3" t="s">
         <v>198</v>
       </c>
-      <c r="L39" s="3" t="s">
+      <c r="M39" s="3" t="s">
         <v>199</v>
-      </c>
-      <c r="M39" s="3" t="s">
-        <v>200</v>
       </c>
       <c r="P39" s="2" t="s">
         <v>35</v>
@@ -5402,7 +5396,7 @@
     </row>
     <row r="40">
       <c r="A40" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B40" s="3" t="s">
         <v>31</v>
@@ -5423,16 +5417,16 @@
         <v>40</v>
       </c>
       <c r="J40" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="K40" s="3" t="s">
         <v>202</v>
       </c>
-      <c r="K40" s="3" t="s">
+      <c r="L40" s="3" t="s">
         <v>203</v>
       </c>
-      <c r="L40" s="3" t="s">
+      <c r="M40" s="3" t="s">
         <v>204</v>
-      </c>
-      <c r="M40" s="3" t="s">
-        <v>205</v>
       </c>
       <c r="P40" s="2" t="s">
         <v>35</v>
@@ -5497,7 +5491,7 @@
     </row>
     <row r="41">
       <c r="A41" s="3" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B41" s="3" t="s">
         <v>31</v>
@@ -5518,13 +5512,13 @@
         <v>40</v>
       </c>
       <c r="J41" s="3" t="s">
+        <v>206</v>
+      </c>
+      <c r="K41" s="3" t="s">
         <v>207</v>
       </c>
-      <c r="K41" s="3" t="s">
+      <c r="L41" s="3" t="s">
         <v>208</v>
-      </c>
-      <c r="L41" s="3" t="s">
-        <v>209</v>
       </c>
       <c r="P41" s="2" t="s">
         <v>35</v>
@@ -5589,7 +5583,7 @@
     </row>
     <row r="42">
       <c r="A42" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B42" s="3" t="s">
         <v>31</v>
@@ -5610,13 +5604,13 @@
         <v>40</v>
       </c>
       <c r="J42" s="3" t="s">
+        <v>210</v>
+      </c>
+      <c r="K42" s="3" t="s">
         <v>211</v>
       </c>
-      <c r="K42" s="3" t="s">
+      <c r="L42" s="3" t="s">
         <v>212</v>
-      </c>
-      <c r="L42" s="3" t="s">
-        <v>213</v>
       </c>
       <c r="P42" s="1" t="s">
         <v>36</v>
@@ -5681,7 +5675,7 @@
     </row>
     <row r="43">
       <c r="A43" s="3" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B43" s="3" t="s">
         <v>38</v>
@@ -5705,16 +5699,16 @@
         <v>6</v>
       </c>
       <c r="J43" s="3" t="s">
+        <v>214</v>
+      </c>
+      <c r="K43" s="3" t="s">
         <v>215</v>
       </c>
-      <c r="K43" s="3" t="s">
+      <c r="L43" s="3" t="s">
+        <v>198</v>
+      </c>
+      <c r="M43" s="3" t="s">
         <v>216</v>
-      </c>
-      <c r="L43" s="3" t="s">
-        <v>199</v>
-      </c>
-      <c r="M43" s="3" t="s">
-        <v>217</v>
       </c>
       <c r="P43" s="2" t="s">
         <v>35</v>
@@ -5779,7 +5773,7 @@
     </row>
     <row r="44">
       <c r="A44" s="3" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B44" s="3" t="s">
         <v>31</v>
@@ -5800,13 +5794,13 @@
         <v>45</v>
       </c>
       <c r="J44" s="3" t="s">
+        <v>218</v>
+      </c>
+      <c r="K44" s="3" t="s">
         <v>219</v>
       </c>
-      <c r="K44" s="3" t="s">
+      <c r="L44" s="3" t="s">
         <v>220</v>
-      </c>
-      <c r="L44" s="3" t="s">
-        <v>221</v>
       </c>
       <c r="P44" s="1" t="s">
         <v>36</v>
@@ -5871,7 +5865,7 @@
     </row>
     <row r="45">
       <c r="A45" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B45" s="3" t="s">
         <v>101</v>
@@ -5895,10 +5889,10 @@
         <v>10</v>
       </c>
       <c r="J45" s="3" t="s">
+        <v>222</v>
+      </c>
+      <c r="K45" s="3" t="s">
         <v>223</v>
-      </c>
-      <c r="K45" s="3" t="s">
-        <v>224</v>
       </c>
       <c r="L45" s="3" t="s">
         <v>141</v>
@@ -5969,7 +5963,7 @@
     </row>
     <row r="46">
       <c r="A46" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B46" s="3" t="s">
         <v>31</v>
@@ -5990,13 +5984,13 @@
         <v>40</v>
       </c>
       <c r="J46" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="K46" s="3" t="s">
         <v>226</v>
       </c>
-      <c r="K46" s="3" t="s">
+      <c r="L46" s="3" t="s">
         <v>227</v>
-      </c>
-      <c r="L46" s="3" t="s">
-        <v>228</v>
       </c>
       <c r="P46" s="2" t="s">
         <v>35</v>
@@ -6061,7 +6055,7 @@
     </row>
     <row r="47">
       <c r="A47" s="3" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B47" s="3" t="s">
         <v>31</v>
@@ -6082,13 +6076,13 @@
         <v>50</v>
       </c>
       <c r="J47" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="K47" s="3" t="s">
         <v>230</v>
       </c>
-      <c r="K47" s="3" t="s">
+      <c r="L47" s="3" t="s">
         <v>231</v>
-      </c>
-      <c r="L47" s="3" t="s">
-        <v>232</v>
       </c>
       <c r="M47" s="3" t="s">
         <v>109</v>
@@ -6156,7 +6150,7 @@
     </row>
     <row r="48">
       <c r="A48" s="3" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B48" s="3" t="s">
         <v>31</v>
@@ -6177,10 +6171,10 @@
         <v>50</v>
       </c>
       <c r="J48" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="K48" s="3" t="s">
         <v>234</v>
-      </c>
-      <c r="K48" s="3" t="s">
-        <v>235</v>
       </c>
       <c r="L48" s="3" t="s">
         <v>113</v>
@@ -6248,13 +6242,13 @@
     </row>
     <row r="49">
       <c r="A49" s="3" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B49" s="3" t="s">
         <v>31</v>
       </c>
       <c r="C49" s="3">
-        <v>200</v>
+        <v>250</v>
       </c>
       <c r="D49" s="3">
         <v>0.25</v>
@@ -6269,16 +6263,13 @@
         <v>50</v>
       </c>
       <c r="J49" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="K49" s="3" t="s">
         <v>237</v>
       </c>
-      <c r="K49" s="3" t="s">
+      <c r="L49" s="3" t="s">
         <v>238</v>
-      </c>
-      <c r="L49" s="3" t="s">
-        <v>239</v>
-      </c>
-      <c r="M49" s="3" t="s">
-        <v>240</v>
       </c>
       <c r="P49" s="1" t="s">
         <v>36</v>
@@ -6343,7 +6334,7 @@
     </row>
     <row r="50">
       <c r="A50" s="3" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="B50" s="3" t="s">
         <v>31</v>
@@ -6364,13 +6355,13 @@
         <v>50</v>
       </c>
       <c r="J50" s="3" t="s">
+        <v>240</v>
+      </c>
+      <c r="K50" s="3" t="s">
+        <v>241</v>
+      </c>
+      <c r="L50" s="3" t="s">
         <v>242</v>
-      </c>
-      <c r="K50" s="3" t="s">
-        <v>243</v>
-      </c>
-      <c r="L50" s="3" t="s">
-        <v>244</v>
       </c>
       <c r="P50" s="1" t="s">
         <v>36</v>
@@ -6435,7 +6426,7 @@
     </row>
     <row r="51">
       <c r="A51" s="3" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="B51" s="3" t="s">
         <v>31</v>
@@ -6456,13 +6447,13 @@
         <v>50</v>
       </c>
       <c r="J51" s="3" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="K51" s="3" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="L51" s="3" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="P51" s="2" t="s">
         <v>35</v>
@@ -6653,13 +6644,13 @@
         <v>22</v>
       </c>
       <c r="AB1" s="4" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="AC1" s="4" t="s">
         <v>25</v>
       </c>
       <c r="AD1" s="4" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="AE1" s="4" t="s">
         <v>26</v>
@@ -6668,12 +6659,12 @@
         <v>28</v>
       </c>
       <c r="AG1" s="4" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>31</v>
@@ -6694,13 +6685,13 @@
         <v>60</v>
       </c>
       <c r="J2" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="K2" s="3" t="s">
         <v>193</v>
       </c>
-      <c r="K2" s="3" t="s">
-        <v>194</v>
-      </c>
       <c r="L2" s="3" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="P2" s="2" t="s">
         <v>35</v>
@@ -6759,7 +6750,7 @@
     </row>
     <row r="3">
       <c r="A3" s="3" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>31</v>
@@ -6783,7 +6774,7 @@
         <v>72</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="L3" s="3" t="s">
         <v>73</v>
@@ -6845,7 +6836,7 @@
     </row>
     <row r="4">
       <c r="A4" s="3" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>31</v>
@@ -6869,13 +6860,13 @@
         <v>32</v>
       </c>
       <c r="K4" s="3" t="s">
+        <v>254</v>
+      </c>
+      <c r="L4" s="3" t="s">
+        <v>255</v>
+      </c>
+      <c r="M4" s="3" t="s">
         <v>256</v>
-      </c>
-      <c r="L4" s="3" t="s">
-        <v>257</v>
-      </c>
-      <c r="M4" s="3" t="s">
-        <v>258</v>
       </c>
       <c r="P4" s="2" t="s">
         <v>35</v>
@@ -6934,7 +6925,7 @@
     </row>
     <row r="5">
       <c r="A5" s="3" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>38</v>
@@ -6961,7 +6952,7 @@
         <v>76</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="L5" s="3" t="s">
         <v>78</v>
@@ -7029,7 +7020,7 @@
     </row>
     <row r="6">
       <c r="A6" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>31</v>
@@ -7118,7 +7109,7 @@
     </row>
     <row r="7">
       <c r="A7" s="3" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>101</v>
@@ -7148,7 +7139,7 @@
         <v>103</v>
       </c>
       <c r="L7" s="3" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="P7" s="1" t="s">
         <v>36</v>
@@ -7207,7 +7198,7 @@
     </row>
     <row r="8">
       <c r="A8" s="3" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>31</v>
@@ -7228,10 +7219,10 @@
         <v>55</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="K8" s="3" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="P8" s="2" t="s">
         <v>35</v>
@@ -7290,7 +7281,7 @@
     </row>
     <row r="9">
       <c r="A9" s="3" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>31</v>
@@ -7311,10 +7302,10 @@
         <v>50</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="K9" s="3" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="L9" s="3" t="s">
         <v>119</v>
@@ -7379,7 +7370,7 @@
     </row>
     <row r="10">
       <c r="A10" s="3" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>31</v>
@@ -7400,13 +7391,13 @@
         <v>50</v>
       </c>
       <c r="J10" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="K10" s="3" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="L10" s="3" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="M10" s="3" t="s">
         <v>118</v>
@@ -7468,7 +7459,7 @@
     </row>
     <row r="11">
       <c r="A11" s="3" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>31</v>
@@ -7489,13 +7480,13 @@
         <v>40</v>
       </c>
       <c r="J11" s="3" t="s">
+        <v>270</v>
+      </c>
+      <c r="K11" s="3" t="s">
+        <v>271</v>
+      </c>
+      <c r="L11" s="3" t="s">
         <v>272</v>
-      </c>
-      <c r="K11" s="3" t="s">
-        <v>273</v>
-      </c>
-      <c r="L11" s="3" t="s">
-        <v>274</v>
       </c>
       <c r="M11" s="3" t="s">
         <v>135</v>
@@ -7557,7 +7548,7 @@
     </row>
     <row r="12">
       <c r="A12" s="3" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>101</v>
@@ -7581,16 +7572,16 @@
         <v>9</v>
       </c>
       <c r="J12" s="3" t="s">
+        <v>274</v>
+      </c>
+      <c r="K12" s="3" t="s">
+        <v>275</v>
+      </c>
+      <c r="L12" s="3" t="s">
         <v>276</v>
       </c>
-      <c r="K12" s="3" t="s">
+      <c r="M12" s="3" t="s">
         <v>277</v>
-      </c>
-      <c r="L12" s="3" t="s">
-        <v>278</v>
-      </c>
-      <c r="M12" s="3" t="s">
-        <v>279</v>
       </c>
       <c r="P12" s="2" t="s">
         <v>35</v>
@@ -7649,7 +7640,7 @@
     </row>
     <row r="13">
       <c r="A13" s="3" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>31</v>
@@ -7738,7 +7729,7 @@
     </row>
     <row r="14">
       <c r="A14" s="3" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>31</v>
@@ -7827,7 +7818,7 @@
     </row>
     <row r="15">
       <c r="A15" s="3" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>31</v>
@@ -7848,19 +7839,19 @@
         <v>40</v>
       </c>
       <c r="J15" s="3" t="s">
+        <v>281</v>
+      </c>
+      <c r="K15" s="3" t="s">
+        <v>282</v>
+      </c>
+      <c r="L15" s="3" t="s">
         <v>283</v>
       </c>
-      <c r="K15" s="3" t="s">
+      <c r="M15" s="3" t="s">
         <v>284</v>
       </c>
-      <c r="L15" s="3" t="s">
+      <c r="N15" s="3" t="s">
         <v>285</v>
-      </c>
-      <c r="M15" s="3" t="s">
-        <v>286</v>
-      </c>
-      <c r="N15" s="3" t="s">
-        <v>287</v>
       </c>
       <c r="O15" s="3" t="s">
         <v>118</v>
@@ -7922,7 +7913,7 @@
     </row>
     <row r="16">
       <c r="A16" s="3" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>31</v>
@@ -7943,13 +7934,13 @@
         <v>45</v>
       </c>
       <c r="J16" s="3" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="K16" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="L16" s="3" t="s">
         <v>180</v>
-      </c>
-      <c r="L16" s="3" t="s">
-        <v>181</v>
       </c>
       <c r="M16" s="3" t="s">
         <v>118</v>
@@ -8011,7 +8002,7 @@
     </row>
     <row r="17">
       <c r="A17" s="3" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>31</v>
@@ -8032,10 +8023,10 @@
         <v>55</v>
       </c>
       <c r="J17" s="3" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="K17" s="3" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="L17" s="3" t="s">
         <v>129</v>
@@ -8100,7 +8091,7 @@
     </row>
     <row r="18">
       <c r="A18" s="3" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>31</v>
@@ -8121,13 +8112,13 @@
         <v>20</v>
       </c>
       <c r="J18" s="3" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="K18" s="3" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="L18" s="3" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="P18" s="2" t="s">
         <v>35</v>
@@ -8186,7 +8177,7 @@
     </row>
     <row r="19">
       <c r="A19" s="3" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>31</v>
@@ -8207,13 +8198,13 @@
         <v>40</v>
       </c>
       <c r="J19" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="K19" s="3" t="s">
         <v>189</v>
       </c>
-      <c r="K19" s="3" t="s">
+      <c r="L19" s="3" t="s">
         <v>190</v>
-      </c>
-      <c r="L19" s="3" t="s">
-        <v>191</v>
       </c>
       <c r="M19" s="3" t="s">
         <v>118</v>
@@ -8275,7 +8266,7 @@
     </row>
     <row r="20">
       <c r="A20" s="3" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>38</v>
@@ -8299,16 +8290,16 @@
         <v>6</v>
       </c>
       <c r="J20" s="3" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="K20" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="L20" s="3" t="s">
+        <v>198</v>
+      </c>
+      <c r="M20" s="3" t="s">
         <v>216</v>
-      </c>
-      <c r="L20" s="3" t="s">
-        <v>199</v>
-      </c>
-      <c r="M20" s="3" t="s">
-        <v>217</v>
       </c>
       <c r="P20" s="2" t="s">
         <v>35</v>
@@ -8367,7 +8358,7 @@
     </row>
     <row r="21">
       <c r="A21" s="3" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>31</v>
@@ -8388,13 +8379,13 @@
         <v>40</v>
       </c>
       <c r="J21" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="K21" s="3" t="s">
         <v>226</v>
       </c>
-      <c r="K21" s="3" t="s">
+      <c r="L21" s="3" t="s">
         <v>227</v>
-      </c>
-      <c r="L21" s="3" t="s">
-        <v>228</v>
       </c>
       <c r="M21" s="3" t="s">
         <v>118</v>
@@ -8456,7 +8447,7 @@
     </row>
     <row r="22">
       <c r="A22" s="3" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>31</v>
@@ -8477,13 +8468,13 @@
         <v>45</v>
       </c>
       <c r="J22" s="3" t="s">
+        <v>299</v>
+      </c>
+      <c r="K22" s="3" t="s">
+        <v>300</v>
+      </c>
+      <c r="L22" s="3" t="s">
         <v>301</v>
-      </c>
-      <c r="K22" s="3" t="s">
-        <v>302</v>
-      </c>
-      <c r="L22" s="3" t="s">
-        <v>303</v>
       </c>
       <c r="M22" s="3" t="s">
         <v>134</v>
@@ -8545,7 +8536,7 @@
     </row>
     <row r="23">
       <c r="A23" s="3" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>31</v>
@@ -8566,16 +8557,16 @@
         <v>42</v>
       </c>
       <c r="J23" s="3" t="s">
+        <v>303</v>
+      </c>
+      <c r="K23" s="3" t="s">
+        <v>304</v>
+      </c>
+      <c r="L23" s="3" t="s">
         <v>305</v>
       </c>
-      <c r="K23" s="3" t="s">
+      <c r="M23" s="3" t="s">
         <v>306</v>
-      </c>
-      <c r="L23" s="3" t="s">
-        <v>307</v>
-      </c>
-      <c r="M23" s="3" t="s">
-        <v>308</v>
       </c>
       <c r="P23" s="2" t="s">
         <v>35</v>
@@ -8634,7 +8625,7 @@
     </row>
     <row r="24">
       <c r="A24" s="3" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>31</v>
@@ -8658,7 +8649,7 @@
         <v>81</v>
       </c>
       <c r="K24" s="3" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="L24" s="3" t="s">
         <v>83</v>
@@ -8723,7 +8714,7 @@
     </row>
     <row r="25">
       <c r="A25" s="3" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>31</v>
@@ -8744,16 +8735,16 @@
         <v>45</v>
       </c>
       <c r="J25" s="3" t="s">
+        <v>310</v>
+      </c>
+      <c r="K25" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="L25" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="M25" s="3" t="s">
         <v>312</v>
-      </c>
-      <c r="K25" s="3" t="s">
-        <v>279</v>
-      </c>
-      <c r="L25" s="3" t="s">
-        <v>313</v>
-      </c>
-      <c r="M25" s="3" t="s">
-        <v>314</v>
       </c>
       <c r="P25" s="2" t="s">
         <v>35</v>
@@ -8812,7 +8803,7 @@
     </row>
     <row r="26">
       <c r="A26" s="3" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="B26" s="3" t="s">
         <v>31</v>
@@ -8833,10 +8824,10 @@
         <v>45</v>
       </c>
       <c r="J26" s="3" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="K26" s="3" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="L26" s="3" t="s">
         <v>113</v>
@@ -8898,7 +8889,7 @@
     </row>
     <row r="27">
       <c r="A27" s="3" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="B27" s="3" t="s">
         <v>31</v>
@@ -8928,7 +8919,7 @@
         <v>55</v>
       </c>
       <c r="M27" s="3" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="P27" s="2" t="s">
         <v>35</v>
@@ -8987,7 +8978,7 @@
     </row>
     <row r="28">
       <c r="A28" s="3" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="B28" s="3" t="s">
         <v>31</v>
@@ -9008,19 +8999,19 @@
         <v>45</v>
       </c>
       <c r="J28" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="K28" s="3" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="L28" s="3" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="M28" s="3" t="s">
         <v>109</v>
       </c>
       <c r="N28" s="3" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="P28" s="2" t="s">
         <v>35</v>
@@ -9079,7 +9070,7 @@
     </row>
     <row r="29">
       <c r="A29" s="3" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="B29" s="3" t="s">
         <v>31</v>
@@ -9100,16 +9091,16 @@
         <v>45</v>
       </c>
       <c r="J29" s="3" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="K29" s="3" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="L29" s="3" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="M29" s="3" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="P29" s="2" t="s">
         <v>35</v>
@@ -9273,16 +9264,16 @@
         <v>19</v>
       </c>
       <c r="U1" s="4" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="V1" s="4" t="s">
         <v>21</v>
       </c>
       <c r="W1" s="4" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="X1" s="4" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="Y1" s="4" t="s">
         <v>26</v>
@@ -9290,7 +9281,7 @@
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>31</v>
@@ -9311,16 +9302,16 @@
         <v>35</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="K2" s="3" t="s">
         <v>93</v>
       </c>
       <c r="L2" s="3" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="M2" s="3" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="P2" s="2" t="s">
         <v>35</v>
@@ -9355,7 +9346,7 @@
     </row>
     <row r="3">
       <c r="A3" s="3" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>31</v>
@@ -9376,13 +9367,13 @@
         <v>40</v>
       </c>
       <c r="J3" s="3" t="s">
+        <v>330</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>331</v>
+      </c>
+      <c r="L3" s="3" t="s">
         <v>332</v>
-      </c>
-      <c r="K3" s="3" t="s">
-        <v>333</v>
-      </c>
-      <c r="L3" s="3" t="s">
-        <v>334</v>
       </c>
       <c r="P3" s="2" t="s">
         <v>35</v>
@@ -9417,7 +9408,7 @@
     </row>
     <row r="4">
       <c r="A4" s="3" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>101</v>
@@ -9441,19 +9432,19 @@
         <v>8</v>
       </c>
       <c r="J4" s="3" t="s">
+        <v>334</v>
+      </c>
+      <c r="K4" s="3" t="s">
+        <v>335</v>
+      </c>
+      <c r="L4" s="3" t="s">
         <v>336</v>
       </c>
-      <c r="K4" s="3" t="s">
-        <v>337</v>
-      </c>
-      <c r="L4" s="3" t="s">
-        <v>338</v>
-      </c>
       <c r="M4" s="3" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="N4" s="3" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="P4" s="2" t="s">
         <v>35</v>
@@ -9488,7 +9479,7 @@
     </row>
     <row r="5">
       <c r="A5" s="3" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>31</v>
@@ -9509,16 +9500,16 @@
         <v>35</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="L5" s="3" t="s">
         <v>111</v>
       </c>
       <c r="M5" s="3" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="P5" s="2" t="s">
         <v>35</v>
@@ -9553,7 +9544,7 @@
     </row>
     <row r="6">
       <c r="A6" s="3" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>31</v>
@@ -9577,13 +9568,13 @@
         <v>32</v>
       </c>
       <c r="K6" s="3" t="s">
+        <v>254</v>
+      </c>
+      <c r="L6" s="3" t="s">
         <v>256</v>
       </c>
-      <c r="L6" s="3" t="s">
-        <v>258</v>
-      </c>
       <c r="M6" s="3" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="P6" s="1" t="s">
         <v>36</v>
@@ -9618,7 +9609,7 @@
     </row>
     <row r="7">
       <c r="A7" s="3" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>31</v>
@@ -9639,16 +9630,16 @@
         <v>30</v>
       </c>
       <c r="J7" s="3" t="s">
+        <v>343</v>
+      </c>
+      <c r="K7" s="3" t="s">
+        <v>344</v>
+      </c>
+      <c r="L7" s="3" t="s">
         <v>345</v>
       </c>
-      <c r="K7" s="3" t="s">
-        <v>346</v>
-      </c>
-      <c r="L7" s="3" t="s">
-        <v>347</v>
-      </c>
       <c r="M7" s="3" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="P7" s="1" t="s">
         <v>36</v>
@@ -9683,7 +9674,7 @@
     </row>
     <row r="8">
       <c r="A8" s="3" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>38</v>
@@ -9707,16 +9698,16 @@
         <v>7</v>
       </c>
       <c r="J8" s="3" t="s">
+        <v>347</v>
+      </c>
+      <c r="K8" s="3" t="s">
+        <v>348</v>
+      </c>
+      <c r="L8" s="3" t="s">
         <v>349</v>
       </c>
-      <c r="K8" s="3" t="s">
+      <c r="M8" s="3" t="s">
         <v>350</v>
-      </c>
-      <c r="L8" s="3" t="s">
-        <v>351</v>
-      </c>
-      <c r="M8" s="3" t="s">
-        <v>352</v>
       </c>
       <c r="P8" s="1" t="s">
         <v>36</v>
@@ -9751,7 +9742,7 @@
     </row>
     <row r="9">
       <c r="A9" s="3" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>31</v>
@@ -9772,16 +9763,16 @@
         <v>45</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="K9" s="3" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="L9" s="3" t="s">
         <v>129</v>
       </c>
       <c r="M9" s="3" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="N9" s="3" t="s">
         <v>131</v>
@@ -9819,7 +9810,7 @@
     </row>
     <row r="10">
       <c r="A10" s="3" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>38</v>
@@ -9843,13 +9834,13 @@
         <v>10</v>
       </c>
       <c r="J10" s="3" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="K10" s="3" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="L10" s="3" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="M10" s="3" t="s">
         <v>135</v>
@@ -9887,7 +9878,7 @@
     </row>
     <row r="11">
       <c r="A11" s="3" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>101</v>
@@ -9911,13 +9902,13 @@
         <v>9</v>
       </c>
       <c r="J11" s="3" t="s">
+        <v>356</v>
+      </c>
+      <c r="K11" s="3" t="s">
+        <v>357</v>
+      </c>
+      <c r="L11" s="3" t="s">
         <v>358</v>
-      </c>
-      <c r="K11" s="3" t="s">
-        <v>359</v>
-      </c>
-      <c r="L11" s="3" t="s">
-        <v>360</v>
       </c>
       <c r="P11" s="2" t="s">
         <v>35</v>
@@ -9952,7 +9943,7 @@
     </row>
     <row r="12">
       <c r="A12" s="3" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>38</v>
@@ -9979,16 +9970,16 @@
         <v>141</v>
       </c>
       <c r="K12" s="3" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="L12" s="3" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="M12" s="3" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="N12" s="3" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="P12" s="2" t="s">
         <v>35</v>
@@ -10023,7 +10014,7 @@
     </row>
     <row r="13">
       <c r="A13" s="3" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>31</v>
@@ -10091,7 +10082,7 @@
     </row>
     <row r="14">
       <c r="A14" s="3" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>31</v>
@@ -10112,13 +10103,13 @@
         <v>50</v>
       </c>
       <c r="J14" s="3" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="K14" s="3" t="s">
         <v>63</v>
       </c>
       <c r="L14" s="3" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="M14" s="3" t="s">
         <v>65</v>
@@ -10159,7 +10150,7 @@
     </row>
     <row r="15">
       <c r="A15" s="3" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>31</v>
@@ -10180,16 +10171,16 @@
         <v>30</v>
       </c>
       <c r="J15" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="K15" s="3" t="s">
         <v>169</v>
       </c>
-      <c r="K15" s="3" t="s">
+      <c r="L15" s="3" t="s">
         <v>170</v>
       </c>
-      <c r="L15" s="3" t="s">
+      <c r="M15" s="3" t="s">
         <v>171</v>
-      </c>
-      <c r="M15" s="3" t="s">
-        <v>172</v>
       </c>
       <c r="P15" s="1" t="s">
         <v>36</v>
@@ -10224,7 +10215,7 @@
     </row>
     <row r="16">
       <c r="A16" s="3" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>31</v>
@@ -10245,19 +10236,19 @@
         <v>35</v>
       </c>
       <c r="J16" s="3" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="K16" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="L16" s="3" t="s">
         <v>175</v>
       </c>
-      <c r="L16" s="3" t="s">
-        <v>176</v>
-      </c>
       <c r="M16" s="3" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="N16" s="3" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="P16" s="2" t="s">
         <v>35</v>
@@ -10292,7 +10283,7 @@
     </row>
     <row r="17">
       <c r="A17" s="3" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>31</v>
@@ -10322,7 +10313,7 @@
         <v>70</v>
       </c>
       <c r="M17" s="3" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="P17" s="2" t="s">
         <v>35</v>
@@ -10357,7 +10348,7 @@
     </row>
     <row r="18">
       <c r="A18" s="3" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>31</v>
@@ -10378,16 +10369,16 @@
         <v>40</v>
       </c>
       <c r="J18" s="3" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="K18" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="L18" s="3" t="s">
         <v>180</v>
       </c>
-      <c r="L18" s="3" t="s">
-        <v>181</v>
-      </c>
       <c r="M18" s="3" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="P18" s="1" t="s">
         <v>36</v>
@@ -10422,7 +10413,7 @@
     </row>
     <row r="19">
       <c r="A19" s="3" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>31</v>
@@ -10443,16 +10434,16 @@
         <v>35</v>
       </c>
       <c r="J19" s="3" t="s">
+        <v>374</v>
+      </c>
+      <c r="K19" s="3" t="s">
+        <v>375</v>
+      </c>
+      <c r="L19" s="3" t="s">
         <v>376</v>
       </c>
-      <c r="K19" s="3" t="s">
+      <c r="M19" s="3" t="s">
         <v>377</v>
-      </c>
-      <c r="L19" s="3" t="s">
-        <v>378</v>
-      </c>
-      <c r="M19" s="3" t="s">
-        <v>379</v>
       </c>
       <c r="P19" s="1" t="s">
         <v>36</v>
@@ -10487,7 +10478,7 @@
     </row>
     <row r="20">
       <c r="A20" s="3" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>31</v>
@@ -10508,16 +10499,16 @@
         <v>45</v>
       </c>
       <c r="J20" s="3" t="s">
+        <v>379</v>
+      </c>
+      <c r="K20" s="3" t="s">
+        <v>380</v>
+      </c>
+      <c r="L20" s="3" t="s">
         <v>381</v>
       </c>
-      <c r="K20" s="3" t="s">
+      <c r="M20" s="3" t="s">
         <v>382</v>
-      </c>
-      <c r="L20" s="3" t="s">
-        <v>383</v>
-      </c>
-      <c r="M20" s="3" t="s">
-        <v>384</v>
       </c>
       <c r="P20" s="1" t="s">
         <v>36</v>
@@ -10552,7 +10543,7 @@
     </row>
     <row r="21">
       <c r="A21" s="3" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>31</v>
@@ -10573,16 +10564,16 @@
         <v>35</v>
       </c>
       <c r="J21" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="K21" s="3" t="s">
         <v>193</v>
       </c>
-      <c r="K21" s="3" t="s">
+      <c r="L21" s="3" t="s">
         <v>194</v>
       </c>
-      <c r="L21" s="3" t="s">
-        <v>195</v>
-      </c>
       <c r="M21" s="3" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="P21" s="1" t="s">
         <v>36</v>
@@ -10617,7 +10608,7 @@
     </row>
     <row r="22">
       <c r="A22" s="3" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>31</v>
@@ -10638,16 +10629,16 @@
         <v>30</v>
       </c>
       <c r="J22" s="3" t="s">
+        <v>385</v>
+      </c>
+      <c r="K22" s="3" t="s">
+        <v>386</v>
+      </c>
+      <c r="L22" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="K22" s="3" t="s">
-        <v>388</v>
-      </c>
-      <c r="L22" s="3" t="s">
-        <v>389</v>
-      </c>
       <c r="M22" s="3" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="P22" s="1" t="s">
         <v>36</v>
@@ -10682,7 +10673,7 @@
     </row>
     <row r="23">
       <c r="A23" s="3" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>38</v>
@@ -10709,7 +10700,7 @@
         <v>76</v>
       </c>
       <c r="K23" s="3" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="L23" s="3" t="s">
         <v>78</v>
@@ -10718,7 +10709,7 @@
         <v>79</v>
       </c>
       <c r="N23" s="3" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="P23" s="2" t="s">
         <v>35</v>
@@ -10753,7 +10744,7 @@
     </row>
     <row r="24">
       <c r="A24" s="3" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>31</v>
@@ -10774,13 +10765,13 @@
         <v>20</v>
       </c>
       <c r="J24" s="3" t="s">
+        <v>391</v>
+      </c>
+      <c r="K24" s="3" t="s">
+        <v>392</v>
+      </c>
+      <c r="L24" s="3" t="s">
         <v>393</v>
-      </c>
-      <c r="K24" s="3" t="s">
-        <v>394</v>
-      </c>
-      <c r="L24" s="3" t="s">
-        <v>395</v>
       </c>
       <c r="P24" s="2" t="s">
         <v>35</v>
@@ -10815,7 +10806,7 @@
     </row>
     <row r="25">
       <c r="A25" s="3" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>31</v>
@@ -10836,16 +10827,16 @@
         <v>30</v>
       </c>
       <c r="J25" s="3" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="K25" s="3" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="L25" s="3" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="M25" s="3" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="P25" s="2" t="s">
         <v>35</v>
@@ -10880,7 +10871,7 @@
     </row>
     <row r="26">
       <c r="A26" s="3" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="B26" s="3" t="s">
         <v>31</v>
@@ -10901,13 +10892,13 @@
         <v>35</v>
       </c>
       <c r="J26" s="3" t="s">
+        <v>397</v>
+      </c>
+      <c r="K26" s="3" t="s">
+        <v>398</v>
+      </c>
+      <c r="L26" s="3" t="s">
         <v>399</v>
-      </c>
-      <c r="K26" s="3" t="s">
-        <v>400</v>
-      </c>
-      <c r="L26" s="3" t="s">
-        <v>401</v>
       </c>
       <c r="P26" s="1" t="s">
         <v>36</v>
@@ -10942,7 +10933,7 @@
     </row>
     <row r="27">
       <c r="A27" s="3" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="B27" s="3" t="s">
         <v>31</v>
@@ -10963,16 +10954,16 @@
         <v>35</v>
       </c>
       <c r="J27" s="3" t="s">
+        <v>401</v>
+      </c>
+      <c r="K27" s="3" t="s">
+        <v>402</v>
+      </c>
+      <c r="L27" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="M27" s="3" t="s">
         <v>403</v>
-      </c>
-      <c r="K27" s="3" t="s">
-        <v>404</v>
-      </c>
-      <c r="L27" s="3" t="s">
-        <v>228</v>
-      </c>
-      <c r="M27" s="3" t="s">
-        <v>405</v>
       </c>
       <c r="P27" s="1" t="s">
         <v>36</v>
@@ -11007,7 +10998,7 @@
     </row>
     <row r="28">
       <c r="A28" s="3" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="B28" s="3" t="s">
         <v>38</v>
@@ -11168,16 +11159,16 @@
         <v>11</v>
       </c>
       <c r="Q1" s="4" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="R1" s="4" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="S1" s="4" t="s">
         <v>17</v>
       </c>
       <c r="T1" s="4" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="U1" s="4" t="s">
         <v>19</v>
@@ -11194,7 +11185,7 @@
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>38</v>
@@ -11218,7 +11209,7 @@
         <v>4</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="P2" s="2" t="s">
         <v>35</v>
@@ -11250,7 +11241,7 @@
     </row>
     <row r="3">
       <c r="A3" s="3" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>31</v>
@@ -11271,10 +11262,10 @@
         <v>39</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
       <c r="L3" s="3" t="s">
         <v>94</v>
@@ -11309,7 +11300,7 @@
     </row>
     <row r="4">
       <c r="A4" s="3" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>38</v>
@@ -11333,13 +11324,13 @@
         <v>9</v>
       </c>
       <c r="J4" s="3" t="s">
+        <v>414</v>
+      </c>
+      <c r="K4" s="3" t="s">
+        <v>415</v>
+      </c>
+      <c r="L4" s="3" t="s">
         <v>416</v>
-      </c>
-      <c r="K4" s="3" t="s">
-        <v>417</v>
-      </c>
-      <c r="L4" s="3" t="s">
-        <v>418</v>
       </c>
       <c r="M4" s="3" t="s">
         <v>99</v>
@@ -11374,7 +11365,7 @@
     </row>
     <row r="5">
       <c r="A5" s="3" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>101</v>
@@ -11398,16 +11389,16 @@
         <v>12</v>
       </c>
       <c r="J5" s="3" t="s">
+        <v>334</v>
+      </c>
+      <c r="K5" s="3" t="s">
+        <v>335</v>
+      </c>
+      <c r="L5" s="3" t="s">
         <v>336</v>
       </c>
-      <c r="K5" s="3" t="s">
-        <v>337</v>
-      </c>
-      <c r="L5" s="3" t="s">
-        <v>338</v>
-      </c>
       <c r="M5" s="3" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="P5" s="1" t="s">
         <v>36</v>
@@ -11439,7 +11430,7 @@
     </row>
     <row r="6">
       <c r="A6" s="3" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>31</v>
@@ -11460,10 +11451,10 @@
         <v>45</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="K6" s="3" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="L6" s="3" t="s">
         <v>113</v>
@@ -11498,7 +11489,7 @@
     </row>
     <row r="7">
       <c r="A7" s="3" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>31</v>
@@ -11528,7 +11519,7 @@
         <v>34</v>
       </c>
       <c r="M7" s="3" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="P7" s="1" t="s">
         <v>36</v>
@@ -11560,7 +11551,7 @@
     </row>
     <row r="8">
       <c r="A8" s="3" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>31</v>
@@ -11581,16 +11572,16 @@
         <v>45</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="K8" s="3" t="s">
         <v>118</v>
       </c>
       <c r="L8" s="3" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="M8" s="3" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="P8" s="1" t="s">
         <v>36</v>
@@ -11622,7 +11613,7 @@
     </row>
     <row r="9">
       <c r="A9" s="3" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>38</v>
@@ -11646,16 +11637,16 @@
         <v>8</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
       <c r="K9" s="3" t="s">
         <v>40</v>
       </c>
       <c r="L9" s="3" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="M9" s="3" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="P9" s="1" t="s">
         <v>36</v>
@@ -11687,7 +11678,7 @@
     </row>
     <row r="10">
       <c r="A10" s="3" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>31</v>
@@ -11708,13 +11699,13 @@
         <v>45</v>
       </c>
       <c r="J10" s="3" t="s">
+        <v>431</v>
+      </c>
+      <c r="K10" s="3" t="s">
+        <v>432</v>
+      </c>
+      <c r="L10" s="3" t="s">
         <v>433</v>
-      </c>
-      <c r="K10" s="3" t="s">
-        <v>434</v>
-      </c>
-      <c r="L10" s="3" t="s">
-        <v>435</v>
       </c>
       <c r="M10" s="3" t="s">
         <v>125</v>
@@ -11749,7 +11740,7 @@
     </row>
     <row r="11">
       <c r="A11" s="3" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>31</v>
@@ -11770,16 +11761,16 @@
         <v>45</v>
       </c>
       <c r="J11" s="3" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="K11" s="3" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="L11" s="3" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
       <c r="M11" s="3" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="N11" s="3" t="s">
         <v>131</v>
@@ -11814,7 +11805,7 @@
     </row>
     <row r="12">
       <c r="A12" s="3" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>31</v>
@@ -11835,10 +11826,10 @@
         <v>37</v>
       </c>
       <c r="J12" s="3" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
       <c r="K12" s="3" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="L12" s="3" t="s">
         <v>49</v>
@@ -11876,7 +11867,7 @@
     </row>
     <row r="13">
       <c r="A13" s="3" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>31</v>
@@ -11938,7 +11929,7 @@
     </row>
     <row r="14">
       <c r="A14" s="3" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>101</v>
@@ -11962,13 +11953,13 @@
         <v>12</v>
       </c>
       <c r="J14" s="3" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="K14" s="3" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
       <c r="L14" s="3" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="P14" s="2" t="s">
         <v>35</v>
@@ -12000,7 +11991,7 @@
     </row>
     <row r="15">
       <c r="A15" s="3" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>38</v>
@@ -12024,16 +12015,16 @@
         <v>9</v>
       </c>
       <c r="J15" s="3" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="K15" s="3" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
       <c r="L15" s="3" t="s">
         <v>143</v>
       </c>
       <c r="M15" s="3" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="P15" s="2" t="s">
         <v>35</v>
@@ -12065,7 +12056,7 @@
     </row>
     <row r="16">
       <c r="A16" s="3" t="s">
-        <v>448</v>
+        <v>446</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>31</v>
@@ -12092,7 +12083,7 @@
         <v>53</v>
       </c>
       <c r="L16" s="3" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="M16" s="3" t="s">
         <v>55</v>
@@ -12130,7 +12121,7 @@
     </row>
     <row r="17">
       <c r="A17" s="3" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>31</v>
@@ -12151,13 +12142,13 @@
         <v>40</v>
       </c>
       <c r="J17" s="3" t="s">
+        <v>449</v>
+      </c>
+      <c r="K17" s="3" t="s">
+        <v>450</v>
+      </c>
+      <c r="L17" s="3" t="s">
         <v>451</v>
-      </c>
-      <c r="K17" s="3" t="s">
-        <v>452</v>
-      </c>
-      <c r="L17" s="3" t="s">
-        <v>453</v>
       </c>
       <c r="M17" s="3" t="s">
         <v>153</v>
@@ -12192,7 +12183,7 @@
     </row>
     <row r="18">
       <c r="A18" s="3" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>31</v>
@@ -12213,16 +12204,16 @@
         <v>41</v>
       </c>
       <c r="J18" s="3" t="s">
+        <v>453</v>
+      </c>
+      <c r="K18" s="3" t="s">
+        <v>454</v>
+      </c>
+      <c r="L18" s="3" t="s">
         <v>455</v>
       </c>
-      <c r="K18" s="3" t="s">
+      <c r="M18" s="3" t="s">
         <v>456</v>
-      </c>
-      <c r="L18" s="3" t="s">
-        <v>457</v>
-      </c>
-      <c r="M18" s="3" t="s">
-        <v>458</v>
       </c>
       <c r="N18" s="3" t="s">
         <v>162</v>
@@ -12257,7 +12248,7 @@
     </row>
     <row r="19">
       <c r="A19" s="3" t="s">
-        <v>459</v>
+        <v>457</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>31</v>
@@ -12278,16 +12269,16 @@
         <v>39</v>
       </c>
       <c r="J19" s="3" t="s">
+        <v>458</v>
+      </c>
+      <c r="K19" s="3" t="s">
+        <v>459</v>
+      </c>
+      <c r="L19" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="M19" s="3" t="s">
         <v>460</v>
-      </c>
-      <c r="K19" s="3" t="s">
-        <v>461</v>
-      </c>
-      <c r="L19" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="M19" s="3" t="s">
-        <v>462</v>
       </c>
       <c r="N19" s="3" t="s">
         <v>66</v>
@@ -12322,7 +12313,7 @@
     </row>
     <row r="20">
       <c r="A20" s="3" t="s">
-        <v>463</v>
+        <v>461</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>31</v>
@@ -12343,16 +12334,16 @@
         <v>45</v>
       </c>
       <c r="J20" s="3" t="s">
+        <v>462</v>
+      </c>
+      <c r="K20" s="3" t="s">
+        <v>463</v>
+      </c>
+      <c r="L20" s="3" t="s">
         <v>464</v>
       </c>
-      <c r="K20" s="3" t="s">
-        <v>465</v>
-      </c>
-      <c r="L20" s="3" t="s">
-        <v>466</v>
-      </c>
       <c r="M20" s="3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="P20" s="1" t="s">
         <v>36</v>
@@ -12384,7 +12375,7 @@
     </row>
     <row r="21">
       <c r="A21" s="3" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>31</v>
@@ -12405,13 +12396,13 @@
         <v>41</v>
       </c>
       <c r="J21" s="3" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="K21" s="3" t="s">
-        <v>468</v>
+        <v>466</v>
       </c>
       <c r="L21" s="3" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
       <c r="P21" s="2" t="s">
         <v>35</v>
@@ -12443,7 +12434,7 @@
     </row>
     <row r="22">
       <c r="A22" s="3" t="s">
-        <v>470</v>
+        <v>468</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>31</v>
@@ -12470,10 +12461,10 @@
         <v>69</v>
       </c>
       <c r="L22" s="3" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
       <c r="M22" s="3" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
       <c r="P22" s="2" t="s">
         <v>35</v>
@@ -12505,7 +12496,7 @@
     </row>
     <row r="23">
       <c r="A23" s="3" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>31</v>
@@ -12526,13 +12517,13 @@
         <v>45</v>
       </c>
       <c r="J23" s="3" t="s">
+        <v>472</v>
+      </c>
+      <c r="K23" s="3" t="s">
+        <v>473</v>
+      </c>
+      <c r="L23" s="3" t="s">
         <v>474</v>
-      </c>
-      <c r="K23" s="3" t="s">
-        <v>475</v>
-      </c>
-      <c r="L23" s="3" t="s">
-        <v>476</v>
       </c>
       <c r="P23" s="2" t="s">
         <v>35</v>
@@ -12564,7 +12555,7 @@
     </row>
     <row r="24">
       <c r="A24" s="3" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>31</v>
@@ -12585,7 +12576,7 @@
         <v>32</v>
       </c>
       <c r="J24" s="3" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
       <c r="P24" s="1" t="s">
         <v>36</v>
@@ -12617,7 +12608,7 @@
     </row>
     <row r="25">
       <c r="A25" s="3" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>31</v>
@@ -12638,16 +12629,16 @@
         <v>31</v>
       </c>
       <c r="J25" s="3" t="s">
+        <v>478</v>
+      </c>
+      <c r="K25" s="3" t="s">
+        <v>479</v>
+      </c>
+      <c r="L25" s="3" t="s">
         <v>480</v>
       </c>
-      <c r="K25" s="3" t="s">
-        <v>481</v>
-      </c>
-      <c r="L25" s="3" t="s">
-        <v>482</v>
-      </c>
       <c r="M25" s="3" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="P25" s="1" t="s">
         <v>36</v>
@@ -12679,7 +12670,7 @@
     </row>
     <row r="26">
       <c r="A26" s="3" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
       <c r="B26" s="3" t="s">
         <v>31</v>
@@ -12738,7 +12729,7 @@
     </row>
     <row r="27">
       <c r="A27" s="3" t="s">
-        <v>484</v>
+        <v>482</v>
       </c>
       <c r="B27" s="3" t="s">
         <v>31</v>
@@ -12759,13 +12750,13 @@
         <v>45</v>
       </c>
       <c r="J27" s="3" t="s">
+        <v>483</v>
+      </c>
+      <c r="K27" s="3" t="s">
+        <v>484</v>
+      </c>
+      <c r="L27" s="3" t="s">
         <v>485</v>
-      </c>
-      <c r="K27" s="3" t="s">
-        <v>486</v>
-      </c>
-      <c r="L27" s="3" t="s">
-        <v>487</v>
       </c>
       <c r="P27" s="1" t="s">
         <v>36</v>
@@ -12797,7 +12788,7 @@
     </row>
     <row r="28">
       <c r="A28" s="3" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="B28" s="3" t="s">
         <v>31</v>
@@ -12818,13 +12809,13 @@
         <v>45</v>
       </c>
       <c r="J28" s="3" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="K28" s="3" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
       <c r="L28" s="3" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
       <c r="P28" s="2" t="s">
         <v>35</v>
@@ -12856,7 +12847,7 @@
     </row>
     <row r="29">
       <c r="A29" s="3" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
       <c r="B29" s="3" t="s">
         <v>31</v>
@@ -12877,16 +12868,16 @@
         <v>50</v>
       </c>
       <c r="J29" s="3" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
       <c r="K29" s="3" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="L29" s="3" t="s">
-        <v>493</v>
+        <v>491</v>
       </c>
       <c r="M29" s="3" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="P29" s="2" t="s">
         <v>35</v>
@@ -12918,7 +12909,7 @@
     </row>
     <row r="30">
       <c r="A30" s="3" t="s">
-        <v>494</v>
+        <v>492</v>
       </c>
       <c r="B30" s="3" t="s">
         <v>38</v>
@@ -12948,10 +12939,10 @@
         <v>77</v>
       </c>
       <c r="L30" s="3" t="s">
-        <v>495</v>
+        <v>493</v>
       </c>
       <c r="M30" s="3" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
       <c r="P30" s="2" t="s">
         <v>35</v>
@@ -12983,7 +12974,7 @@
     </row>
     <row r="31">
       <c r="A31" s="3" t="s">
-        <v>497</v>
+        <v>495</v>
       </c>
       <c r="B31" s="3" t="s">
         <v>31</v>
@@ -13004,13 +12995,13 @@
         <v>25</v>
       </c>
       <c r="J31" s="3" t="s">
-        <v>498</v>
+        <v>496</v>
       </c>
       <c r="K31" s="3" t="s">
         <v>82</v>
       </c>
       <c r="L31" s="3" t="s">
-        <v>499</v>
+        <v>497</v>
       </c>
       <c r="P31" s="2" t="s">
         <v>35</v>
@@ -13042,7 +13033,7 @@
     </row>
     <row r="32">
       <c r="A32" s="3" t="s">
-        <v>500</v>
+        <v>498</v>
       </c>
       <c r="B32" s="3" t="s">
         <v>31</v>
@@ -13063,13 +13054,13 @@
         <v>45</v>
       </c>
       <c r="J32" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="K32" s="3" t="s">
-        <v>501</v>
+        <v>499</v>
       </c>
       <c r="L32" s="3" t="s">
-        <v>502</v>
+        <v>500</v>
       </c>
       <c r="P32" s="2" t="s">
         <v>35</v>
@@ -13101,7 +13092,7 @@
     </row>
     <row r="33">
       <c r="A33" s="3" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
       <c r="B33" s="3" t="s">
         <v>31</v>
@@ -13122,13 +13113,13 @@
         <v>45</v>
       </c>
       <c r="J33" s="3" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
       <c r="K33" s="3" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="L33" s="3" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="P33" s="1" t="s">
         <v>36</v>
@@ -13160,7 +13151,7 @@
     </row>
     <row r="34">
       <c r="A34" s="3" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
       <c r="B34" s="3" t="s">
         <v>31</v>
@@ -13181,13 +13172,13 @@
         <v>50</v>
       </c>
       <c r="J34" s="3" t="s">
+        <v>505</v>
+      </c>
+      <c r="K34" s="3" t="s">
+        <v>506</v>
+      </c>
+      <c r="L34" s="3" t="s">
         <v>507</v>
-      </c>
-      <c r="K34" s="3" t="s">
-        <v>508</v>
-      </c>
-      <c r="L34" s="3" t="s">
-        <v>509</v>
       </c>
       <c r="P34" s="1" t="s">
         <v>36</v>
@@ -13219,7 +13210,7 @@
     </row>
     <row r="35">
       <c r="A35" s="3" t="s">
-        <v>510</v>
+        <v>508</v>
       </c>
       <c r="B35" s="3" t="s">
         <v>31</v>
@@ -13240,13 +13231,13 @@
         <v>45</v>
       </c>
       <c r="J35" s="3" t="s">
-        <v>511</v>
+        <v>509</v>
       </c>
       <c r="K35" s="3" t="s">
-        <v>512</v>
+        <v>510</v>
       </c>
       <c r="L35" s="3" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="P35" s="2" t="s">
         <v>35</v>
@@ -13278,7 +13269,7 @@
     </row>
     <row r="36">
       <c r="A36" s="3" t="s">
-        <v>513</v>
+        <v>511</v>
       </c>
       <c r="B36" s="3" t="s">
         <v>38</v>
@@ -13442,24 +13433,24 @@
         <v>16</v>
       </c>
       <c r="S1" s="4" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="T1" s="4" t="s">
-        <v>514</v>
+        <v>512</v>
       </c>
       <c r="U1" s="4" t="s">
         <v>26</v>
       </c>
       <c r="V1" s="4" t="s">
-        <v>515</v>
+        <v>513</v>
       </c>
       <c r="W1" s="4" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>38</v>
@@ -13483,16 +13474,16 @@
         <v>6</v>
       </c>
       <c r="J2" s="3" t="s">
+        <v>515</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>516</v>
+      </c>
+      <c r="L2" s="3" t="s">
         <v>517</v>
       </c>
-      <c r="K2" s="3" t="s">
+      <c r="M2" s="3" t="s">
         <v>518</v>
-      </c>
-      <c r="L2" s="3" t="s">
-        <v>519</v>
-      </c>
-      <c r="M2" s="3" t="s">
-        <v>520</v>
       </c>
       <c r="P2" s="1" t="s">
         <v>36</v>
@@ -13521,7 +13512,7 @@
     </row>
     <row r="3">
       <c r="A3" s="3" t="s">
-        <v>521</v>
+        <v>519</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>31</v>
@@ -13542,13 +13533,13 @@
         <v>20</v>
       </c>
       <c r="J3" s="3" t="s">
+        <v>520</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>521</v>
+      </c>
+      <c r="L3" s="3" t="s">
         <v>522</v>
-      </c>
-      <c r="K3" s="3" t="s">
-        <v>523</v>
-      </c>
-      <c r="L3" s="3" t="s">
-        <v>524</v>
       </c>
       <c r="P3" s="1" t="s">
         <v>36</v>

</xml_diff>